<commit_message>
Deployed 3e436dc with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -16,9 +16,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track Record" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipeline Detail'!$A$3:$AG$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipeline Detail'!$A$3:$AC$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Distress Documentation'!$A$3:$O$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Geographic Targeting'!$A$3:$H$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Geographic Targeting'!$A$3:$H$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Impact Projections'!$A$3:$R$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Investor Commitments'!$A$3:$H$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Track Record'!$A$3:$F$7</definedName>
@@ -223,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -291,6 +291,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -299,26 +302,35 @@
     <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -834,7 +846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -862,7 +874,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>CY2025  |  Prepared: August 15, 2026  |  Readiness Grade: A (86.6/100)</t>
+          <t>CY2025  |  Prepared: August 16, 2026  |  Readiness Grade: A (86.6/100)</t>
         </is>
       </c>
     </row>
@@ -920,7 +932,7 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -998,7 +1010,7 @@
         <v>100</v>
       </c>
       <c r="D18" s="17" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="19" ht="17" customHeight="1">
@@ -1050,7 +1062,7 @@
         <v>100</v>
       </c>
       <c r="D22" s="17" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="23" ht="17" customHeight="1">
@@ -1081,22 +1093,29 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="24" t="inlineStr">
-        <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-15</t>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>READINESS SCORE BREAKDOWN — weights are this tool's own unsourced judgement (eligibility quality 25%; distress concentration 25%; geographic diversity 15%; impact metrics 20%; validation pass rate 10%; completeness 5%); the CDFI Fund publishes no such weighting and this score does not predict an award outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="25" t="inlineStr">
+        <is>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-16</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="33">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A27:F27"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="C10:D10"/>
@@ -1122,6 +1141,7 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1147,42 +1167,38 @@
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="39" customWidth="1" min="11" max="11"/>
     <col width="29" customWidth="1" min="12" max="12"/>
     <col width="25" customWidth="1" min="13" max="13"/>
     <col width="23" customWidth="1" min="14" max="14"/>
     <col width="21" customWidth="1" min="15" max="15"/>
     <col width="25" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="19" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="32" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
-    <col width="23" customWidth="1" min="25" max="25"/>
-    <col width="30" customWidth="1" min="26" max="26"/>
-    <col width="21" customWidth="1" min="27" max="27"/>
-    <col width="19" customWidth="1" min="28" max="28"/>
-    <col width="22" customWidth="1" min="29" max="29"/>
-    <col width="15" customWidth="1" min="30" max="30"/>
-    <col width="16" customWidth="1" min="31" max="31"/>
-    <col width="25" customWidth="1" min="32" max="32"/>
-    <col width="14" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="32" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="21" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="15" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="25" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Appendix A: Pipeline Detail</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-15</t>
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1255,7 @@
       </c>
       <c r="K3" s="14" t="inlineStr">
         <is>
-          <t>NMTC Native Area (Y/N)</t>
+          <t>NMTC Native Area (CDE-declared, Y/N)</t>
         </is>
       </c>
       <c r="L3" s="14" t="inlineStr">
@@ -1274,80 +1290,60 @@
       </c>
       <c r="R3" s="14" t="inlineStr">
         <is>
-          <t>QLICI A Loan ($)</t>
+          <t>Total QLICI ($)</t>
         </is>
       </c>
       <c r="S3" s="14" t="inlineStr">
         <is>
-          <t>QLICI B Loan ($)</t>
+          <t>Leverage Loan ($)</t>
         </is>
       </c>
       <c r="T3" s="14" t="inlineStr">
         <is>
-          <t>Leverage Loan ($)</t>
+          <t>Total NMTCs ($)</t>
         </is>
       </c>
       <c r="U3" s="14" t="inlineStr">
         <is>
-          <t>Total NMTCs ($)</t>
+          <t>Estimated Investor Equity ($)</t>
         </is>
       </c>
       <c r="V3" s="14" t="inlineStr">
         <is>
-          <t>Estimated Investor Equity ($)</t>
+          <t>CDE Fee ($)</t>
         </is>
       </c>
       <c r="W3" s="14" t="inlineStr">
         <is>
-          <t>CDE Fee ($)</t>
+          <t>Construction Start</t>
         </is>
       </c>
       <c r="X3" s="14" t="inlineStr">
         <is>
-          <t>Senior Debt ($)</t>
+          <t>Operations Start</t>
         </is>
       </c>
       <c r="Y3" s="14" t="inlineStr">
         <is>
-          <t>Subordinate Debt ($)</t>
+          <t>Closing Target Date</t>
         </is>
       </c>
       <c r="Z3" s="14" t="inlineStr">
         <is>
-          <t>Annual Operating Budget ($)</t>
+          <t>Jobs Created</t>
         </is>
       </c>
       <c r="AA3" s="14" t="inlineStr">
         <is>
-          <t>Construction Start</t>
+          <t>Jobs Retained</t>
         </is>
       </c>
       <c r="AB3" s="14" t="inlineStr">
         <is>
-          <t>Operations Start</t>
+          <t>Affordable Units Built</t>
         </is>
       </c>
       <c r="AC3" s="14" t="inlineStr">
-        <is>
-          <t>Closing Target Date</t>
-        </is>
-      </c>
-      <c r="AD3" s="14" t="inlineStr">
-        <is>
-          <t>Jobs Created</t>
-        </is>
-      </c>
-      <c r="AE3" s="14" t="inlineStr">
-        <is>
-          <t>Jobs Retained</t>
-        </is>
-      </c>
-      <c r="AF3" s="14" t="inlineStr">
-        <is>
-          <t>Affordable Units Built</t>
-        </is>
-      </c>
-      <c r="AG3" s="14" t="inlineStr">
         <is>
           <t>Square Feet</t>
         </is>
@@ -1425,56 +1421,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P4" s="27" t="n">
+      <c r="P4" s="28" t="n">
         <v>12500000</v>
       </c>
       <c r="Q4" s="28" t="n">
         <v>8500000</v>
       </c>
       <c r="R4" s="28" t="n">
-        <v>1700000</v>
+        <v>8500000</v>
       </c>
       <c r="S4" s="28" t="n">
-        <v>6800000</v>
+        <v>5748550</v>
       </c>
       <c r="T4" s="28" t="n">
-        <v>6800000</v>
+        <v>3315000</v>
       </c>
       <c r="U4" s="28" t="n">
-        <v>3315000</v>
+        <v>2751450</v>
       </c>
       <c r="V4" s="28" t="n">
-        <v>2751450</v>
-      </c>
-      <c r="W4" s="28" t="n">
         <v>212500</v>
       </c>
-      <c r="X4" s="28" t="n">
-        <v>8048550</v>
-      </c>
-      <c r="Y4" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="28" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="AA4" s="5" t="inlineStr"/>
-      <c r="AB4" s="5" t="inlineStr"/>
-      <c r="AC4" s="5" t="inlineStr">
+      <c r="W4" s="5" t="inlineStr"/>
+      <c r="X4" s="5" t="inlineStr"/>
+      <c r="Y4" s="5" t="inlineStr">
         <is>
           <t>2025-09-30</t>
         </is>
       </c>
-      <c r="AD4" s="27" t="n">
+      <c r="Z4" s="29" t="n">
         <v>52</v>
       </c>
-      <c r="AE4" s="27" t="n">
+      <c r="AA4" s="29" t="n">
         <v>18</v>
       </c>
-      <c r="AF4" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG4" s="27" t="n">
+      <c r="AB4" s="29" t="n">
+        <v/>
+      </c>
+      <c r="AC4" s="29" t="n">
         <v>24000</v>
       </c>
     </row>
@@ -1550,56 +1534,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P5" s="29" t="n">
+      <c r="P5" s="30" t="n">
         <v>9800000</v>
       </c>
       <c r="Q5" s="30" t="n">
         <v>7000000</v>
       </c>
       <c r="R5" s="30" t="n">
-        <v>1400000</v>
+        <v>7000000</v>
       </c>
       <c r="S5" s="30" t="n">
-        <v>5600000</v>
+        <v>4734100</v>
       </c>
       <c r="T5" s="30" t="n">
-        <v>5600000</v>
+        <v>2730000</v>
       </c>
       <c r="U5" s="30" t="n">
-        <v>2730000</v>
+        <v>2265900</v>
       </c>
       <c r="V5" s="30" t="n">
-        <v>2265900</v>
-      </c>
-      <c r="W5" s="30" t="n">
         <v>175000</v>
       </c>
-      <c r="X5" s="30" t="n">
-        <v>6134100</v>
-      </c>
-      <c r="Y5" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="30" t="n">
-        <v>784000</v>
-      </c>
-      <c r="AA5" s="7" t="inlineStr"/>
-      <c r="AB5" s="7" t="inlineStr"/>
-      <c r="AC5" s="7" t="inlineStr">
+      <c r="W5" s="7" t="inlineStr"/>
+      <c r="X5" s="7" t="inlineStr"/>
+      <c r="Y5" s="7" t="inlineStr">
         <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="AD5" s="29" t="n">
+      <c r="Z5" s="31" t="n">
         <v>38</v>
       </c>
-      <c r="AE5" s="29" t="n">
+      <c r="AA5" s="31" t="n">
         <v>22</v>
       </c>
-      <c r="AF5" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG5" s="29" t="n">
+      <c r="AB5" s="31" t="n">
+        <v/>
+      </c>
+      <c r="AC5" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1675,56 +1647,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P6" s="27" t="n">
+      <c r="P6" s="28" t="n">
         <v>7200000</v>
       </c>
       <c r="Q6" s="28" t="n">
         <v>5000000</v>
       </c>
       <c r="R6" s="28" t="n">
-        <v>1000000</v>
+        <v>5000000</v>
       </c>
       <c r="S6" s="28" t="n">
-        <v>4000000</v>
+        <v>3381500</v>
       </c>
       <c r="T6" s="28" t="n">
-        <v>4000000</v>
+        <v>1950000</v>
       </c>
       <c r="U6" s="28" t="n">
-        <v>1950000</v>
+        <v>1618500</v>
       </c>
       <c r="V6" s="28" t="n">
-        <v>1618500</v>
-      </c>
-      <c r="W6" s="28" t="n">
         <v>125000</v>
       </c>
-      <c r="X6" s="28" t="n">
-        <v>4581500</v>
-      </c>
-      <c r="Y6" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="28" t="n">
-        <v>576000</v>
-      </c>
-      <c r="AA6" s="5" t="inlineStr"/>
-      <c r="AB6" s="5" t="inlineStr"/>
-      <c r="AC6" s="5" t="inlineStr">
+      <c r="W6" s="5" t="inlineStr"/>
+      <c r="X6" s="5" t="inlineStr"/>
+      <c r="Y6" s="5" t="inlineStr">
         <is>
           <t>2025-08-31</t>
         </is>
       </c>
-      <c r="AD6" s="27" t="n">
+      <c r="Z6" s="29" t="n">
         <v>65</v>
       </c>
-      <c r="AE6" s="27" t="n">
+      <c r="AA6" s="29" t="n">
         <v>8</v>
       </c>
-      <c r="AF6" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG6" s="27" t="n">
+      <c r="AB6" s="29" t="n">
+        <v/>
+      </c>
+      <c r="AC6" s="29" t="n">
         <v>18000</v>
       </c>
     </row>
@@ -1800,56 +1760,44 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="P7" s="29" t="n">
+      <c r="P7" s="30" t="n">
         <v>6000000</v>
       </c>
       <c r="Q7" s="30" t="n">
         <v>4500000</v>
       </c>
       <c r="R7" s="30" t="n">
-        <v>900000</v>
+        <v>4500000</v>
       </c>
       <c r="S7" s="30" t="n">
-        <v>3600000</v>
+        <v>3043350</v>
       </c>
       <c r="T7" s="30" t="n">
-        <v>3600000</v>
+        <v>1755000</v>
       </c>
       <c r="U7" s="30" t="n">
-        <v>1755000</v>
+        <v>1456650</v>
       </c>
       <c r="V7" s="30" t="n">
-        <v>1456650</v>
-      </c>
-      <c r="W7" s="30" t="n">
         <v>112500</v>
       </c>
-      <c r="X7" s="30" t="n">
-        <v>3643350</v>
-      </c>
-      <c r="Y7" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="30" t="n">
-        <v>480000</v>
-      </c>
-      <c r="AA7" s="7" t="inlineStr"/>
-      <c r="AB7" s="7" t="inlineStr"/>
-      <c r="AC7" s="7" t="inlineStr">
+      <c r="W7" s="7" t="inlineStr"/>
+      <c r="X7" s="7" t="inlineStr"/>
+      <c r="Y7" s="7" t="inlineStr">
         <is>
           <t>2025-11-30</t>
         </is>
       </c>
-      <c r="AD7" s="29" t="n">
+      <c r="Z7" s="31" t="n">
         <v>80</v>
       </c>
-      <c r="AE7" s="29" t="n">
+      <c r="AA7" s="31" t="n">
         <v>25</v>
       </c>
-      <c r="AF7" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG7" s="29" t="n">
+      <c r="AB7" s="31" t="n">
+        <v/>
+      </c>
+      <c r="AC7" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1925,56 +1873,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P8" s="27" t="n">
+      <c r="P8" s="28" t="n">
         <v>10000000</v>
       </c>
       <c r="Q8" s="28" t="n">
         <v>7500000</v>
       </c>
       <c r="R8" s="28" t="n">
-        <v>1500000</v>
+        <v>7500000</v>
       </c>
       <c r="S8" s="28" t="n">
-        <v>6000000</v>
+        <v>5072250</v>
       </c>
       <c r="T8" s="28" t="n">
-        <v>6000000</v>
+        <v>2925000</v>
       </c>
       <c r="U8" s="28" t="n">
-        <v>2925000</v>
+        <v>2427750</v>
       </c>
       <c r="V8" s="28" t="n">
-        <v>2427750</v>
-      </c>
-      <c r="W8" s="28" t="n">
         <v>187500</v>
       </c>
-      <c r="X8" s="28" t="n">
-        <v>6072250</v>
-      </c>
-      <c r="Y8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z8" s="28" t="n">
-        <v>800000</v>
-      </c>
-      <c r="AA8" s="5" t="inlineStr"/>
-      <c r="AB8" s="5" t="inlineStr"/>
-      <c r="AC8" s="5" t="inlineStr">
+      <c r="W8" s="5" t="inlineStr"/>
+      <c r="X8" s="5" t="inlineStr"/>
+      <c r="Y8" s="5" t="inlineStr">
         <is>
           <t>2026-01-31</t>
         </is>
       </c>
-      <c r="AD8" s="27" t="n">
+      <c r="Z8" s="29" t="n">
         <v>42</v>
       </c>
-      <c r="AE8" s="27" t="n">
+      <c r="AA8" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="AF8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG8" s="27" t="n">
+      <c r="AB8" s="29" t="n">
+        <v/>
+      </c>
+      <c r="AC8" s="29" t="n">
         <v>20000</v>
       </c>
     </row>
@@ -2050,56 +1986,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P9" s="29" t="n">
+      <c r="P9" s="30" t="n">
         <v>14000000</v>
       </c>
       <c r="Q9" s="30" t="n">
         <v>9000000</v>
       </c>
       <c r="R9" s="30" t="n">
-        <v>1800000</v>
+        <v>9000000</v>
       </c>
       <c r="S9" s="30" t="n">
-        <v>7200000</v>
+        <v>6086700</v>
       </c>
       <c r="T9" s="30" t="n">
-        <v>7200000</v>
+        <v>3510000</v>
       </c>
       <c r="U9" s="30" t="n">
-        <v>3510000</v>
+        <v>2913300</v>
       </c>
       <c r="V9" s="30" t="n">
-        <v>2913300</v>
-      </c>
-      <c r="W9" s="30" t="n">
         <v>225000</v>
       </c>
-      <c r="X9" s="30" t="n">
-        <v>9286700</v>
-      </c>
-      <c r="Y9" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z9" s="30" t="n">
-        <v>1120000</v>
-      </c>
-      <c r="AA9" s="7" t="inlineStr"/>
-      <c r="AB9" s="7" t="inlineStr"/>
-      <c r="AC9" s="7" t="inlineStr">
+      <c r="W9" s="7" t="inlineStr"/>
+      <c r="X9" s="7" t="inlineStr"/>
+      <c r="Y9" s="7" t="inlineStr">
         <is>
           <t>2025-10-31</t>
         </is>
       </c>
-      <c r="AD9" s="29" t="n">
+      <c r="Z9" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="AE9" s="29" t="n">
+      <c r="AA9" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="AF9" s="29" t="n">
+      <c r="AB9" s="31" t="n">
         <v>72</v>
       </c>
-      <c r="AG9" s="29" t="n">
+      <c r="AC9" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2175,56 +2099,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P10" s="27" t="n">
+      <c r="P10" s="28" t="n">
         <v>5500000</v>
       </c>
       <c r="Q10" s="28" t="n">
         <v>4000000</v>
       </c>
       <c r="R10" s="28" t="n">
-        <v>800000</v>
+        <v>4000000</v>
       </c>
       <c r="S10" s="28" t="n">
-        <v>3200000</v>
+        <v>2705200</v>
       </c>
       <c r="T10" s="28" t="n">
-        <v>3200000</v>
+        <v>1560000</v>
       </c>
       <c r="U10" s="28" t="n">
-        <v>1560000</v>
+        <v>1294800</v>
       </c>
       <c r="V10" s="28" t="n">
-        <v>1294800</v>
-      </c>
-      <c r="W10" s="28" t="n">
         <v>100000</v>
       </c>
-      <c r="X10" s="28" t="n">
-        <v>3405200</v>
-      </c>
-      <c r="Y10" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z10" s="28" t="n">
-        <v>440000</v>
-      </c>
-      <c r="AA10" s="5" t="inlineStr"/>
-      <c r="AB10" s="5" t="inlineStr"/>
-      <c r="AC10" s="5" t="inlineStr">
+      <c r="W10" s="5" t="inlineStr"/>
+      <c r="X10" s="5" t="inlineStr"/>
+      <c r="Y10" s="5" t="inlineStr">
         <is>
           <t>2025-09-15</t>
         </is>
       </c>
-      <c r="AD10" s="27" t="n">
+      <c r="Z10" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="AE10" s="27" t="n">
+      <c r="AA10" s="29" t="n">
         <v>10</v>
       </c>
-      <c r="AF10" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG10" s="27" t="n">
+      <c r="AB10" s="29" t="n">
+        <v/>
+      </c>
+      <c r="AC10" s="29" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -2300,56 +2212,44 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="P11" s="29" t="n">
+      <c r="P11" s="30" t="n">
         <v>11000000</v>
       </c>
       <c r="Q11" s="30" t="n">
         <v>8000000</v>
       </c>
       <c r="R11" s="30" t="n">
-        <v>1600000</v>
+        <v>8000000</v>
       </c>
       <c r="S11" s="30" t="n">
-        <v>6400000</v>
+        <v>5410400</v>
       </c>
       <c r="T11" s="30" t="n">
-        <v>6400000</v>
+        <v>3120000</v>
       </c>
       <c r="U11" s="30" t="n">
-        <v>3120000</v>
+        <v>2589600</v>
       </c>
       <c r="V11" s="30" t="n">
-        <v>2589600</v>
-      </c>
-      <c r="W11" s="30" t="n">
         <v>200000</v>
       </c>
-      <c r="X11" s="30" t="n">
-        <v>6810400</v>
-      </c>
-      <c r="Y11" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z11" s="30" t="n">
-        <v>880000</v>
-      </c>
-      <c r="AA11" s="7" t="inlineStr"/>
-      <c r="AB11" s="7" t="inlineStr"/>
-      <c r="AC11" s="7" t="inlineStr">
+      <c r="W11" s="7" t="inlineStr"/>
+      <c r="X11" s="7" t="inlineStr"/>
+      <c r="Y11" s="7" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
       </c>
-      <c r="AD11" s="29" t="n">
+      <c r="Z11" s="31" t="n">
         <v>55</v>
       </c>
-      <c r="AE11" s="29" t="n">
+      <c r="AA11" s="31" t="n">
         <v>20</v>
       </c>
-      <c r="AF11" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG11" s="29" t="n">
+      <c r="AB11" s="31" t="n">
+        <v/>
+      </c>
+      <c r="AC11" s="31" t="n">
         <v>22000</v>
       </c>
     </row>
@@ -2425,56 +2325,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P12" s="27" t="n">
+      <c r="P12" s="28" t="n">
         <v>8200000</v>
       </c>
       <c r="Q12" s="28" t="n">
         <v>6000000</v>
       </c>
       <c r="R12" s="28" t="n">
-        <v>1200000</v>
+        <v>6000000</v>
       </c>
       <c r="S12" s="28" t="n">
-        <v>4800000</v>
+        <v>4057800</v>
       </c>
       <c r="T12" s="28" t="n">
-        <v>4800000</v>
+        <v>2340000</v>
       </c>
       <c r="U12" s="28" t="n">
-        <v>2340000</v>
+        <v>1942200</v>
       </c>
       <c r="V12" s="28" t="n">
-        <v>1942200</v>
-      </c>
-      <c r="W12" s="28" t="n">
         <v>150000</v>
       </c>
-      <c r="X12" s="28" t="n">
-        <v>5057800</v>
-      </c>
-      <c r="Y12" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z12" s="28" t="n">
-        <v>656000</v>
-      </c>
-      <c r="AA12" s="5" t="inlineStr"/>
-      <c r="AB12" s="5" t="inlineStr"/>
-      <c r="AC12" s="5" t="inlineStr">
+      <c r="W12" s="5" t="inlineStr"/>
+      <c r="X12" s="5" t="inlineStr"/>
+      <c r="Y12" s="5" t="inlineStr">
         <is>
           <t>2025-11-15</t>
         </is>
       </c>
-      <c r="AD12" s="27" t="n">
+      <c r="Z12" s="29" t="n">
         <v>35</v>
       </c>
-      <c r="AE12" s="27" t="n">
+      <c r="AA12" s="29" t="n">
         <v>8</v>
       </c>
-      <c r="AF12" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG12" s="27" t="n">
+      <c r="AB12" s="29" t="n">
+        <v/>
+      </c>
+      <c r="AC12" s="29" t="n">
         <v>16000</v>
       </c>
     </row>
@@ -2550,56 +2438,44 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="P13" s="29" t="n">
+      <c r="P13" s="30" t="n">
         <v>4800000</v>
       </c>
       <c r="Q13" s="30" t="n">
         <v>3500000</v>
       </c>
       <c r="R13" s="30" t="n">
-        <v>700000</v>
+        <v>3500000</v>
       </c>
       <c r="S13" s="30" t="n">
-        <v>2800000</v>
+        <v>2367050</v>
       </c>
       <c r="T13" s="30" t="n">
-        <v>2800000</v>
+        <v>1365000</v>
       </c>
       <c r="U13" s="30" t="n">
-        <v>1365000</v>
+        <v>1132950</v>
       </c>
       <c r="V13" s="30" t="n">
-        <v>1132950</v>
-      </c>
-      <c r="W13" s="30" t="n">
         <v>87500</v>
       </c>
-      <c r="X13" s="30" t="n">
-        <v>2967050</v>
-      </c>
-      <c r="Y13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z13" s="30" t="n">
-        <v>384000</v>
-      </c>
-      <c r="AA13" s="7" t="inlineStr"/>
-      <c r="AB13" s="7" t="inlineStr"/>
-      <c r="AC13" s="7" t="inlineStr">
+      <c r="W13" s="7" t="inlineStr"/>
+      <c r="X13" s="7" t="inlineStr"/>
+      <c r="Y13" s="7" t="inlineStr">
         <is>
           <t>2025-08-15</t>
         </is>
       </c>
-      <c r="AD13" s="29" t="n">
+      <c r="Z13" s="31" t="n">
         <v>90</v>
       </c>
-      <c r="AE13" s="29" t="n">
+      <c r="AA13" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="AF13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG13" s="29" t="n">
+      <c r="AB13" s="31" t="n">
+        <v/>
+      </c>
+      <c r="AC13" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2675,56 +2551,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P14" s="27" t="n">
+      <c r="P14" s="28" t="n">
         <v>13500000</v>
       </c>
       <c r="Q14" s="28" t="n">
         <v>9500000</v>
       </c>
       <c r="R14" s="28" t="n">
-        <v>1900000</v>
+        <v>9500000</v>
       </c>
       <c r="S14" s="28" t="n">
-        <v>7600000</v>
+        <v>6424850</v>
       </c>
       <c r="T14" s="28" t="n">
-        <v>7600000</v>
+        <v>3705000</v>
       </c>
       <c r="U14" s="28" t="n">
-        <v>3705000</v>
+        <v>3075150</v>
       </c>
       <c r="V14" s="28" t="n">
-        <v>3075150</v>
-      </c>
-      <c r="W14" s="28" t="n">
         <v>237500</v>
       </c>
-      <c r="X14" s="28" t="n">
-        <v>8524850</v>
-      </c>
-      <c r="Y14" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="28" t="n">
-        <v>1080000</v>
-      </c>
-      <c r="AA14" s="5" t="inlineStr"/>
-      <c r="AB14" s="5" t="inlineStr"/>
-      <c r="AC14" s="5" t="inlineStr">
+      <c r="W14" s="5" t="inlineStr"/>
+      <c r="X14" s="5" t="inlineStr"/>
+      <c r="Y14" s="5" t="inlineStr">
         <is>
           <t>2026-02-28</t>
         </is>
       </c>
-      <c r="AD14" s="27" t="n">
+      <c r="Z14" s="29" t="n">
         <v>12</v>
       </c>
-      <c r="AE14" s="27" t="n">
+      <c r="AA14" s="29" t="n">
         <v>4</v>
       </c>
-      <c r="AF14" s="27" t="n">
+      <c r="AB14" s="29" t="n">
         <v>64</v>
       </c>
-      <c r="AG14" s="27" t="n">
+      <c r="AC14" s="29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2800,56 +2664,44 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="P15" s="29" t="n">
+      <c r="P15" s="30" t="n">
         <v>5000000</v>
       </c>
       <c r="Q15" s="30" t="n">
         <v>3800000</v>
       </c>
       <c r="R15" s="30" t="n">
-        <v>760000</v>
+        <v>3800000</v>
       </c>
       <c r="S15" s="30" t="n">
-        <v>3040000</v>
+        <v>2569940</v>
       </c>
       <c r="T15" s="30" t="n">
-        <v>3040000</v>
+        <v>1482000</v>
       </c>
       <c r="U15" s="30" t="n">
-        <v>1482000</v>
+        <v>1230060</v>
       </c>
       <c r="V15" s="30" t="n">
-        <v>1230060</v>
-      </c>
-      <c r="W15" s="30" t="n">
         <v>95000</v>
       </c>
-      <c r="X15" s="30" t="n">
-        <v>3009940</v>
-      </c>
-      <c r="Y15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z15" s="30" t="n">
-        <v>400000</v>
-      </c>
-      <c r="AA15" s="7" t="inlineStr"/>
-      <c r="AB15" s="7" t="inlineStr"/>
-      <c r="AC15" s="7" t="inlineStr">
+      <c r="W15" s="7" t="inlineStr"/>
+      <c r="X15" s="7" t="inlineStr"/>
+      <c r="Y15" s="7" t="inlineStr">
         <is>
           <t>2025-10-15</t>
         </is>
       </c>
-      <c r="AD15" s="29" t="n">
+      <c r="Z15" s="31" t="n">
         <v>22</v>
       </c>
-      <c r="AE15" s="29" t="n">
+      <c r="AA15" s="31" t="n">
         <v>6</v>
       </c>
-      <c r="AF15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG15" s="29" t="n">
+      <c r="AB15" s="31" t="n">
+        <v/>
+      </c>
+      <c r="AC15" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2871,7 +2723,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>2800 Freedom Dr</t>
+          <t>2810 Freedom Dr</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -2887,7 +2739,7 @@
       <c r="G16" s="5" t="inlineStr"/>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>37119001900</t>
+          <t>37119004200</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -2897,7 +2749,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Deep Distress</t>
+          <t>Severely Distressed</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2925,56 +2777,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P16" s="27" t="n">
+      <c r="P16" s="28" t="n">
         <v>7500000</v>
       </c>
       <c r="Q16" s="28" t="n">
         <v>5500000</v>
       </c>
       <c r="R16" s="28" t="n">
-        <v>1100000</v>
+        <v>5500000</v>
       </c>
       <c r="S16" s="28" t="n">
-        <v>4400000</v>
+        <v>3719650</v>
       </c>
       <c r="T16" s="28" t="n">
-        <v>4400000</v>
+        <v>2145000</v>
       </c>
       <c r="U16" s="28" t="n">
-        <v>2145000</v>
+        <v>1780350</v>
       </c>
       <c r="V16" s="28" t="n">
-        <v>1780350</v>
-      </c>
-      <c r="W16" s="28" t="n">
         <v>137500</v>
       </c>
-      <c r="X16" s="28" t="n">
-        <v>4619650</v>
-      </c>
-      <c r="Y16" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z16" s="28" t="n">
-        <v>600000</v>
-      </c>
-      <c r="AA16" s="5" t="inlineStr"/>
-      <c r="AB16" s="5" t="inlineStr"/>
-      <c r="AC16" s="5" t="inlineStr">
+      <c r="W16" s="5" t="inlineStr"/>
+      <c r="X16" s="5" t="inlineStr"/>
+      <c r="Y16" s="5" t="inlineStr">
         <is>
           <t>2025-12-31</t>
         </is>
       </c>
-      <c r="AD16" s="27" t="n">
+      <c r="Z16" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="AE16" s="27" t="n">
+      <c r="AA16" s="29" t="n">
         <v>12</v>
       </c>
-      <c r="AF16" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG16" s="27" t="n">
+      <c r="AB16" s="29" t="n">
+        <v/>
+      </c>
+      <c r="AC16" s="29" t="n">
         <v>14000</v>
       </c>
     </row>
@@ -3050,56 +2890,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P17" s="29" t="n">
+      <c r="P17" s="30" t="n">
         <v>9000000</v>
       </c>
       <c r="Q17" s="30" t="n">
         <v>6500000</v>
       </c>
       <c r="R17" s="30" t="n">
-        <v>1300000</v>
+        <v>6500000</v>
       </c>
       <c r="S17" s="30" t="n">
-        <v>5200000</v>
+        <v>4395950</v>
       </c>
       <c r="T17" s="30" t="n">
-        <v>5200000</v>
+        <v>2535000</v>
       </c>
       <c r="U17" s="30" t="n">
-        <v>2535000</v>
+        <v>2104050</v>
       </c>
       <c r="V17" s="30" t="n">
-        <v>2104050</v>
-      </c>
-      <c r="W17" s="30" t="n">
         <v>162500</v>
       </c>
-      <c r="X17" s="30" t="n">
-        <v>5595950</v>
-      </c>
-      <c r="Y17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z17" s="30" t="n">
-        <v>720000</v>
-      </c>
-      <c r="AA17" s="7" t="inlineStr"/>
-      <c r="AB17" s="7" t="inlineStr"/>
-      <c r="AC17" s="7" t="inlineStr">
+      <c r="W17" s="7" t="inlineStr"/>
+      <c r="X17" s="7" t="inlineStr"/>
+      <c r="Y17" s="7" t="inlineStr">
         <is>
           <t>2026-01-15</t>
         </is>
       </c>
-      <c r="AD17" s="29" t="n">
+      <c r="Z17" s="31" t="n">
         <v>48</v>
       </c>
-      <c r="AE17" s="29" t="n">
+      <c r="AA17" s="31" t="n">
         <v>25</v>
       </c>
-      <c r="AF17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG17" s="29" t="n">
+      <c r="AB17" s="31" t="n">
+        <v/>
+      </c>
+      <c r="AC17" s="31" t="n">
         <v>18500</v>
       </c>
     </row>
@@ -3175,56 +3003,44 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="P18" s="27" t="n">
+      <c r="P18" s="28" t="n">
         <v>6500000</v>
       </c>
       <c r="Q18" s="28" t="n">
         <v>5000000</v>
       </c>
       <c r="R18" s="28" t="n">
-        <v>1000000</v>
+        <v>5000000</v>
       </c>
       <c r="S18" s="28" t="n">
-        <v>4000000</v>
+        <v>3381500</v>
       </c>
       <c r="T18" s="28" t="n">
-        <v>4000000</v>
+        <v>1950000</v>
       </c>
       <c r="U18" s="28" t="n">
-        <v>1950000</v>
+        <v>1618500</v>
       </c>
       <c r="V18" s="28" t="n">
-        <v>1618500</v>
-      </c>
-      <c r="W18" s="28" t="n">
         <v>125000</v>
       </c>
-      <c r="X18" s="28" t="n">
-        <v>3881500</v>
-      </c>
-      <c r="Y18" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z18" s="28" t="n">
-        <v>520000</v>
-      </c>
-      <c r="AA18" s="5" t="inlineStr"/>
-      <c r="AB18" s="5" t="inlineStr"/>
-      <c r="AC18" s="5" t="inlineStr">
+      <c r="W18" s="5" t="inlineStr"/>
+      <c r="X18" s="5" t="inlineStr"/>
+      <c r="Y18" s="5" t="inlineStr">
         <is>
           <t>2025-09-30</t>
         </is>
       </c>
-      <c r="AD18" s="27" t="n">
+      <c r="Z18" s="29" t="n">
         <v>110</v>
       </c>
-      <c r="AE18" s="27" t="n">
+      <c r="AA18" s="29" t="n">
         <v>45</v>
       </c>
-      <c r="AF18" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG18" s="27" t="n">
+      <c r="AB18" s="29" t="n">
+        <v/>
+      </c>
+      <c r="AC18" s="29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3300,56 +3116,44 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="P19" s="29" t="n">
+      <c r="P19" s="30" t="n">
         <v>10500000</v>
       </c>
       <c r="Q19" s="30" t="n">
         <v>7500000</v>
       </c>
       <c r="R19" s="30" t="n">
-        <v>1500000</v>
+        <v>7500000</v>
       </c>
       <c r="S19" s="30" t="n">
-        <v>6000000</v>
+        <v>5072250</v>
       </c>
       <c r="T19" s="30" t="n">
-        <v>6000000</v>
+        <v>2925000</v>
       </c>
       <c r="U19" s="30" t="n">
-        <v>2925000</v>
+        <v>2427750</v>
       </c>
       <c r="V19" s="30" t="n">
-        <v>2427750</v>
-      </c>
-      <c r="W19" s="30" t="n">
         <v>187500</v>
       </c>
-      <c r="X19" s="30" t="n">
-        <v>6572250</v>
-      </c>
-      <c r="Y19" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z19" s="30" t="n">
-        <v>840000</v>
-      </c>
-      <c r="AA19" s="7" t="inlineStr"/>
-      <c r="AB19" s="7" t="inlineStr"/>
-      <c r="AC19" s="7" t="inlineStr">
+      <c r="W19" s="7" t="inlineStr"/>
+      <c r="X19" s="7" t="inlineStr"/>
+      <c r="Y19" s="7" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="AD19" s="29" t="n">
+      <c r="Z19" s="31" t="n">
         <v>35</v>
       </c>
-      <c r="AE19" s="29" t="n">
+      <c r="AA19" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="AF19" s="29" t="n">
+      <c r="AB19" s="31" t="n">
         <v>24</v>
       </c>
-      <c r="AG19" s="29" t="n">
+      <c r="AC19" s="31" t="n">
         <v>20000</v>
       </c>
     </row>
@@ -3425,56 +3229,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P20" s="27" t="n">
+      <c r="P20" s="28" t="n">
         <v>4200000</v>
       </c>
       <c r="Q20" s="28" t="n">
         <v>3200000</v>
       </c>
       <c r="R20" s="28" t="n">
-        <v>640000</v>
+        <v>3200000</v>
       </c>
       <c r="S20" s="28" t="n">
-        <v>2560000</v>
+        <v>2164160</v>
       </c>
       <c r="T20" s="28" t="n">
-        <v>2560000</v>
+        <v>1248000</v>
       </c>
       <c r="U20" s="28" t="n">
-        <v>1248000</v>
+        <v>1035840</v>
       </c>
       <c r="V20" s="28" t="n">
-        <v>1035840</v>
-      </c>
-      <c r="W20" s="28" t="n">
         <v>80000</v>
       </c>
-      <c r="X20" s="28" t="n">
-        <v>2524160</v>
-      </c>
-      <c r="Y20" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z20" s="28" t="n">
-        <v>336000</v>
-      </c>
-      <c r="AA20" s="5" t="inlineStr"/>
-      <c r="AB20" s="5" t="inlineStr"/>
-      <c r="AC20" s="5" t="inlineStr">
+      <c r="W20" s="5" t="inlineStr"/>
+      <c r="X20" s="5" t="inlineStr"/>
+      <c r="Y20" s="5" t="inlineStr">
         <is>
           <t>2025-11-30</t>
         </is>
       </c>
-      <c r="AD20" s="27" t="n">
+      <c r="Z20" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="AE20" s="27" t="n">
+      <c r="AA20" s="29" t="n">
         <v>15</v>
       </c>
-      <c r="AF20" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG20" s="27" t="n">
+      <c r="AB20" s="29" t="n">
+        <v/>
+      </c>
+      <c r="AC20" s="29" t="n">
         <v>8000</v>
       </c>
     </row>
@@ -3506,13 +3298,13 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>KS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr"/>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>20091000100</t>
+          <t>29095017800</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
@@ -3550,56 +3342,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P21" s="29" t="n">
+      <c r="P21" s="30" t="n">
         <v>11800000</v>
       </c>
       <c r="Q21" s="30" t="n">
         <v>8500000</v>
       </c>
       <c r="R21" s="30" t="n">
-        <v>1700000</v>
+        <v>8500000</v>
       </c>
       <c r="S21" s="30" t="n">
-        <v>6800000</v>
+        <v>5748550</v>
       </c>
       <c r="T21" s="30" t="n">
-        <v>6800000</v>
+        <v>3315000</v>
       </c>
       <c r="U21" s="30" t="n">
-        <v>3315000</v>
+        <v>2751450</v>
       </c>
       <c r="V21" s="30" t="n">
-        <v>2751450</v>
-      </c>
-      <c r="W21" s="30" t="n">
         <v>212500</v>
       </c>
-      <c r="X21" s="30" t="n">
-        <v>7348550</v>
-      </c>
-      <c r="Y21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z21" s="30" t="n">
-        <v>944000</v>
-      </c>
-      <c r="AA21" s="7" t="inlineStr"/>
-      <c r="AB21" s="7" t="inlineStr"/>
-      <c r="AC21" s="7" t="inlineStr">
+      <c r="W21" s="7" t="inlineStr"/>
+      <c r="X21" s="7" t="inlineStr"/>
+      <c r="Y21" s="7" t="inlineStr">
         <is>
           <t>2026-02-15</t>
         </is>
       </c>
-      <c r="AD21" s="29" t="n">
+      <c r="Z21" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="AE21" s="29" t="n">
+      <c r="AA21" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="AF21" s="29" t="n">
+      <c r="AB21" s="31" t="n">
         <v>56</v>
       </c>
-      <c r="AG21" s="29" t="n">
+      <c r="AC21" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3675,56 +3455,44 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P22" s="27" t="n">
+      <c r="P22" s="28" t="n">
         <v>5800000</v>
       </c>
       <c r="Q22" s="28" t="n">
         <v>4200000</v>
       </c>
       <c r="R22" s="28" t="n">
-        <v>840000</v>
+        <v>4200000</v>
       </c>
       <c r="S22" s="28" t="n">
-        <v>3360000</v>
+        <v>2840460</v>
       </c>
       <c r="T22" s="28" t="n">
-        <v>3360000</v>
+        <v>1638000</v>
       </c>
       <c r="U22" s="28" t="n">
-        <v>1638000</v>
+        <v>1359540</v>
       </c>
       <c r="V22" s="28" t="n">
-        <v>1359540</v>
-      </c>
-      <c r="W22" s="28" t="n">
         <v>105000</v>
       </c>
-      <c r="X22" s="28" t="n">
-        <v>3600460</v>
-      </c>
-      <c r="Y22" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z22" s="28" t="n">
-        <v>464000</v>
-      </c>
-      <c r="AA22" s="5" t="inlineStr"/>
-      <c r="AB22" s="5" t="inlineStr"/>
-      <c r="AC22" s="5" t="inlineStr">
+      <c r="W22" s="5" t="inlineStr"/>
+      <c r="X22" s="5" t="inlineStr"/>
+      <c r="Y22" s="5" t="inlineStr">
         <is>
           <t>2025-10-31</t>
         </is>
       </c>
-      <c r="AD22" s="27" t="n">
+      <c r="Z22" s="29" t="n">
         <v>45</v>
       </c>
-      <c r="AE22" s="27" t="n">
+      <c r="AA22" s="29" t="n">
         <v>8</v>
       </c>
-      <c r="AF22" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG22" s="27" t="n">
+      <c r="AB22" s="29" t="n">
+        <v/>
+      </c>
+      <c r="AC22" s="29" t="n">
         <v>11000</v>
       </c>
     </row>
@@ -3800,135 +3568,113 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="P23" s="29" t="n">
+      <c r="P23" s="30" t="n">
         <v>7800000</v>
       </c>
       <c r="Q23" s="30" t="n">
         <v>5800000</v>
       </c>
       <c r="R23" s="30" t="n">
-        <v>1160000</v>
+        <v>5800000</v>
       </c>
       <c r="S23" s="30" t="n">
-        <v>4640000</v>
+        <v>3922540</v>
       </c>
       <c r="T23" s="30" t="n">
-        <v>4640000</v>
+        <v>2262000</v>
       </c>
       <c r="U23" s="30" t="n">
-        <v>2262000</v>
+        <v>1877460</v>
       </c>
       <c r="V23" s="30" t="n">
-        <v>1877460</v>
-      </c>
-      <c r="W23" s="30" t="n">
         <v>145000</v>
       </c>
-      <c r="X23" s="30" t="n">
-        <v>4762540</v>
-      </c>
-      <c r="Y23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z23" s="30" t="n">
-        <v>624000</v>
-      </c>
-      <c r="AA23" s="7" t="inlineStr"/>
-      <c r="AB23" s="7" t="inlineStr"/>
-      <c r="AC23" s="7" t="inlineStr">
+      <c r="W23" s="7" t="inlineStr"/>
+      <c r="X23" s="7" t="inlineStr"/>
+      <c r="Y23" s="7" t="inlineStr">
         <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="AD23" s="29" t="n">
+      <c r="Z23" s="31" t="n">
         <v>32</v>
       </c>
-      <c r="AE23" s="29" t="n">
+      <c r="AA23" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="AF23" s="29" t="n">
+      <c r="AB23" s="31" t="n">
         <v>18</v>
       </c>
-      <c r="AG23" s="29" t="n">
+      <c r="AC23" s="31" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B24" s="31" t="inlineStr"/>
-      <c r="C24" s="31" t="inlineStr">
+      <c r="B24" s="32" t="inlineStr"/>
+      <c r="C24" s="32" t="inlineStr">
         <is>
           <t>TOTAL (20 projects)</t>
         </is>
       </c>
-      <c r="D24" s="31" t="inlineStr"/>
-      <c r="E24" s="31" t="inlineStr"/>
-      <c r="F24" s="31" t="inlineStr"/>
-      <c r="G24" s="31" t="inlineStr"/>
-      <c r="H24" s="31" t="inlineStr"/>
-      <c r="I24" s="31" t="inlineStr"/>
-      <c r="J24" s="31" t="inlineStr"/>
-      <c r="K24" s="31" t="inlineStr"/>
-      <c r="L24" s="31" t="inlineStr"/>
-      <c r="M24" s="31" t="inlineStr"/>
-      <c r="N24" s="31" t="inlineStr"/>
-      <c r="O24" s="31" t="inlineStr"/>
-      <c r="P24" s="32" t="n">
+      <c r="D24" s="32" t="inlineStr"/>
+      <c r="E24" s="32" t="inlineStr"/>
+      <c r="F24" s="32" t="inlineStr"/>
+      <c r="G24" s="32" t="inlineStr"/>
+      <c r="H24" s="32" t="inlineStr"/>
+      <c r="I24" s="32" t="inlineStr"/>
+      <c r="J24" s="32" t="inlineStr"/>
+      <c r="K24" s="32" t="inlineStr"/>
+      <c r="L24" s="32" t="inlineStr"/>
+      <c r="M24" s="32" t="inlineStr"/>
+      <c r="N24" s="32" t="inlineStr"/>
+      <c r="O24" s="32" t="inlineStr"/>
+      <c r="P24" s="33" t="n">
         <v>170600000</v>
       </c>
       <c r="Q24" s="33" t="n">
         <v>122500000</v>
       </c>
       <c r="R24" s="33" t="n">
-        <v>24500000</v>
+        <v>122500000</v>
       </c>
       <c r="S24" s="33" t="n">
-        <v>98000000</v>
+        <v>82846750</v>
       </c>
       <c r="T24" s="33" t="n">
-        <v>98000000</v>
+        <v>47775000</v>
       </c>
       <c r="U24" s="33" t="n">
-        <v>47775000</v>
+        <v>39653250</v>
       </c>
       <c r="V24" s="33" t="n">
-        <v>39653250</v>
-      </c>
-      <c r="W24" s="33" t="n">
         <v>3062500</v>
       </c>
-      <c r="X24" s="33" t="n">
-        <v>106446750</v>
-      </c>
-      <c r="Y24" s="31" t="inlineStr"/>
-      <c r="Z24" s="33" t="n">
-        <v>13648000</v>
-      </c>
-      <c r="AA24" s="31" t="inlineStr"/>
-      <c r="AB24" s="31" t="inlineStr"/>
-      <c r="AC24" s="31" t="inlineStr"/>
-      <c r="AD24" s="32" t="n">
+      <c r="W24" s="32" t="inlineStr"/>
+      <c r="X24" s="32" t="inlineStr"/>
+      <c r="Y24" s="32" t="inlineStr"/>
+      <c r="Z24" s="34" t="n">
         <v>864</v>
       </c>
-      <c r="AE24" s="32" t="n">
+      <c r="AA24" s="34" t="n">
         <v>298</v>
       </c>
-      <c r="AF24" s="32" t="n">
+      <c r="AB24" s="34" t="n">
         <v>234</v>
       </c>
-      <c r="AG24" s="32" t="n">
+      <c r="AC24" s="34" t="n">
         <v>198500</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:AG24"/>
+  <autoFilter ref="A3:AC24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:AG2"/>
-    <mergeCell ref="A1:AG1"/>
+    <mergeCell ref="A2:AC2"/>
+    <mergeCell ref="A1:AC1"/>
   </mergeCells>
   <conditionalFormatting sqref="J4:J24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -3961,7 +3707,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
     <col width="29" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
@@ -3972,16 +3718,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Appendix B: Distress Documentation</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-15</t>
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
         </is>
       </c>
     </row>
@@ -4023,7 +3769,7 @@
       </c>
       <c r="H3" s="14" t="inlineStr">
         <is>
-          <t>NMTC Native Area</t>
+          <t>NMTC Native Area (CDE-declared)</t>
         </is>
       </c>
       <c r="I3" s="14" t="inlineStr">
@@ -5004,7 +4750,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>37119001900</t>
+          <t>37119004200</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -5014,7 +4760,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Deep Distress</t>
+          <t>Severely Distressed</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -5384,12 +5130,12 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Kansas City, KS</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>20091000100</t>
+          <t>29095017800</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -5603,41 +5349,41 @@
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>SUMMARY</t>
         </is>
       </c>
-      <c r="B24" s="31" t="inlineStr">
+      <c r="B24" s="32" t="inlineStr">
         <is>
           <t>20 total projects</t>
         </is>
       </c>
-      <c r="C24" s="31" t="inlineStr"/>
-      <c r="D24" s="31" t="inlineStr"/>
-      <c r="E24" s="31" t="inlineStr">
+      <c r="C24" s="32" t="inlineStr"/>
+      <c r="D24" s="32" t="inlineStr"/>
+      <c r="E24" s="32" t="inlineStr">
         <is>
           <t>20/20</t>
         </is>
       </c>
-      <c r="F24" s="31" t="inlineStr"/>
-      <c r="G24" s="31" t="inlineStr">
+      <c r="F24" s="32" t="inlineStr"/>
+      <c r="G24" s="32" t="inlineStr">
         <is>
           <t>17/20 (85%)</t>
         </is>
       </c>
-      <c r="H24" s="31" t="inlineStr">
+      <c r="H24" s="32" t="inlineStr">
         <is>
           <t>2/20</t>
         </is>
       </c>
-      <c r="I24" s="31" t="inlineStr"/>
-      <c r="J24" s="31" t="inlineStr"/>
-      <c r="K24" s="31" t="inlineStr"/>
-      <c r="L24" s="31" t="inlineStr"/>
-      <c r="M24" s="31" t="inlineStr"/>
-      <c r="N24" s="31" t="inlineStr"/>
-      <c r="O24" s="31" t="inlineStr"/>
+      <c r="I24" s="32" t="inlineStr"/>
+      <c r="J24" s="32" t="inlineStr"/>
+      <c r="K24" s="32" t="inlineStr"/>
+      <c r="L24" s="32" t="inlineStr"/>
+      <c r="M24" s="32" t="inlineStr"/>
+      <c r="N24" s="32" t="inlineStr"/>
+      <c r="O24" s="32" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:O24"/>
@@ -5655,30 +5401,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC24"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Appendix C: Geographic Targeting</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-15</t>
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
         </is>
       </c>
     </row>
@@ -5710,7 +5456,7 @@
       </c>
       <c r="F3" s="14" t="inlineStr">
         <is>
-          <t>Native Area Projects</t>
+          <t>Native Area Projects (CDE-declared)</t>
         </is>
       </c>
       <c r="G3" s="14" t="inlineStr">
@@ -5730,27 +5476,25 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="B4" s="27" t="n">
+      <c r="B4" s="29" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="28" t="n">
         <v>6500000</v>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>5.3%</t>
-        </is>
-      </c>
-      <c r="E4" s="27" t="n">
+      <c r="D4" s="17" t="n">
+        <v>0.05306122448979592</v>
+      </c>
+      <c r="E4" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="27" t="n">
+      <c r="F4" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="27" t="n">
+      <c r="G4" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="27" t="n">
+      <c r="H4" s="29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5760,27 +5504,25 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="B5" s="29" t="n">
+      <c r="B5" s="31" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="30" t="n">
         <v>4500000</v>
       </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>3.7%</t>
-        </is>
-      </c>
-      <c r="E5" s="29" t="n">
+      <c r="D5" s="19" t="n">
+        <v>0.03673469387755102</v>
+      </c>
+      <c r="E5" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="29" t="n">
+      <c r="F5" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="29" t="n">
+      <c r="G5" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="29" t="n">
+      <c r="H5" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5790,27 +5532,25 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="29" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>4000000</v>
       </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>3.3%</t>
-        </is>
-      </c>
-      <c r="E6" s="27" t="n">
+      <c r="D6" s="17" t="n">
+        <v>0.0326530612244898</v>
+      </c>
+      <c r="E6" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="27" t="n">
+      <c r="H6" s="29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5820,27 +5560,25 @@
           <t>GA</t>
         </is>
       </c>
-      <c r="B7" s="29" t="n">
+      <c r="B7" s="31" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="30" t="n">
         <v>9000000</v>
       </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>7.3%</t>
-        </is>
-      </c>
-      <c r="E7" s="29" t="n">
+      <c r="D7" s="19" t="n">
+        <v>0.07346938775510205</v>
+      </c>
+      <c r="E7" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="29" t="n">
+      <c r="F7" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="29" t="n">
+      <c r="G7" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="29" t="n">
+      <c r="H7" s="31" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5850,27 +5588,25 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
+      <c r="B8" s="29" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>8500000</v>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>6.9%</t>
-        </is>
-      </c>
-      <c r="E8" s="27" t="n">
+      <c r="D8" s="17" t="n">
+        <v>0.06938775510204082</v>
+      </c>
+      <c r="E8" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="27" t="n">
+      <c r="G8" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="27" t="n">
+      <c r="H8" s="29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5880,486 +5616,438 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="B9" s="29" t="n">
+      <c r="B9" s="31" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="30" t="n">
         <v>7500000</v>
       </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>6.1%</t>
-        </is>
-      </c>
-      <c r="E9" s="29" t="n">
+      <c r="D9" s="19" t="n">
+        <v>0.06122448979591837</v>
+      </c>
+      <c r="E9" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="29" t="n">
+      <c r="F9" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="29" t="n">
+      <c r="G9" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="29" t="n">
+      <c r="H9" s="31" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>KS</t>
-        </is>
-      </c>
-      <c r="B10" s="27" t="n">
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>8500000</v>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>6.9%</t>
-        </is>
-      </c>
-      <c r="E10" s="27" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>0.04897959183673469</v>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="G10" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="27" t="n">
-        <v>0</v>
+      <c r="H10" s="29" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>LA</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="n">
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="30" t="n">
-        <v>6000000</v>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>4.9%</t>
-        </is>
-      </c>
-      <c r="E11" s="29" t="n">
+        <v>4200000</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>0.03428571428571429</v>
+      </c>
+      <c r="E11" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="29" t="n">
+      <c r="F11" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="29" t="n">
+      <c r="G11" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="29" t="n">
-        <v>1</v>
+      <c r="H11" s="31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="B12" s="27" t="n">
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>4200000</v>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>3.4%</t>
-        </is>
-      </c>
-      <c r="E12" s="27" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>0.04081632653061224</v>
+      </c>
+      <c r="E12" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="27" t="n">
+      <c r="G12" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="27" t="n">
-        <v>0</v>
+      <c r="H12" s="29" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>MI</t>
-        </is>
-      </c>
-      <c r="B13" s="29" t="n">
-        <v>1</v>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="n">
+        <v>2</v>
       </c>
       <c r="C13" s="30" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>4.1%</t>
-        </is>
-      </c>
-      <c r="E13" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="29" t="n">
+        <v>12300000</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>0.1004081632653061</v>
+      </c>
+      <c r="E13" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="29" t="n">
+      <c r="F13" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="29" t="n">
+      <c r="G13" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="31" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="B14" s="27" t="n">
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>3800000</v>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>3.1%</t>
-        </is>
-      </c>
-      <c r="E14" s="27" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>0.02612244897959184</v>
+      </c>
+      <c r="E14" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="27" t="n">
+      <c r="G14" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="29" t="n">
         <v>0</v>
-      </c>
-      <c r="G14" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="27" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>MS</t>
-        </is>
-      </c>
-      <c r="B15" s="29" t="n">
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="30" t="n">
-        <v>3200000</v>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>2.6%</t>
-        </is>
-      </c>
-      <c r="E15" s="29" t="n">
+        <v>5500000</v>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>0.04489795918367347</v>
+      </c>
+      <c r="E15" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="29" t="n">
+      <c r="F15" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" s="29" t="n">
+      <c r="G15" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="31" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="B16" s="27" t="n">
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="28" t="n">
-        <v>5500000</v>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>4.5%</t>
-        </is>
-      </c>
-      <c r="E16" s="27" t="n">
+        <v>5800000</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>0.0473469387755102</v>
+      </c>
+      <c r="E16" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="27" t="n">
+      <c r="F16" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="27" t="n">
-        <v>0</v>
+      <c r="H16" s="29" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>NM</t>
-        </is>
-      </c>
-      <c r="B17" s="29" t="n">
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="30" t="n">
-        <v>5800000</v>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>4.7%</t>
-        </is>
-      </c>
-      <c r="E17" s="29" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>0.04081632653061224</v>
+      </c>
+      <c r="E17" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="29" t="n">
+      <c r="F17" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="29" t="n">
+      <c r="G17" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="31" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="n">
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="28" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>4.1%</t>
-        </is>
-      </c>
-      <c r="E18" s="27" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="D18" s="17" t="n">
+        <v>0.06122448979591837</v>
+      </c>
+      <c r="E18" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="27" t="n">
+      <c r="F18" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="27" t="n">
+      <c r="G18" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="27" t="n">
-        <v>1</v>
+      <c r="H18" s="29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>OH</t>
-        </is>
-      </c>
-      <c r="B19" s="29" t="n">
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="30" t="n">
-        <v>7500000</v>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>6.1%</t>
-        </is>
-      </c>
-      <c r="E19" s="29" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="D19" s="19" t="n">
+        <v>0.0653061224489796</v>
+      </c>
+      <c r="E19" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="29" t="n">
+      <c r="F19" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="29" t="n">
+      <c r="G19" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="29" t="n">
+      <c r="H19" s="31" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="B20" s="27" t="n">
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="28" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>6.5%</t>
-        </is>
-      </c>
-      <c r="E20" s="27" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <v>0.02857142857142857</v>
+      </c>
+      <c r="E20" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="27" t="n">
+      <c r="F20" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="27" t="n">
+      <c r="G20" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="27" t="n">
+      <c r="H20" s="29" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>TN</t>
-        </is>
-      </c>
-      <c r="B21" s="29" t="n">
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="30" t="n">
-        <v>3500000</v>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>2.9%</t>
-        </is>
-      </c>
-      <c r="E21" s="29" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="D21" s="19" t="n">
+        <v>0.05714285714285714</v>
+      </c>
+      <c r="E21" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="29" t="n">
+      <c r="F21" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="29" t="n">
+      <c r="G21" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="29" t="n">
-        <v>0</v>
+      <c r="H21" s="31" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="B22" s="27" t="n">
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="28" t="n">
-        <v>7000000</v>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>5.7%</t>
-        </is>
-      </c>
-      <c r="E22" s="27" t="n">
+        <v>9500000</v>
+      </c>
+      <c r="D22" s="17" t="n">
+        <v>0.07755102040816327</v>
+      </c>
+      <c r="E22" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="27" t="n">
+      <c r="F22" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="27" t="n">
+      <c r="G22" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="27" t="n">
+      <c r="H22" s="29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="32" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B23" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="C23" s="33" t="n">
+        <v>122500000</v>
+      </c>
+      <c r="D23" s="35" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>WI</t>
-        </is>
-      </c>
-      <c r="B23" s="29" t="n">
+      <c r="E23" s="34" t="n">
+        <v>17</v>
+      </c>
+      <c r="F23" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="30" t="n">
-        <v>9500000</v>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>7.8%</t>
-        </is>
-      </c>
-      <c r="E23" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="29" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B24" s="32" t="n">
-        <v>20</v>
-      </c>
-      <c r="C24" s="33" t="n">
-        <v>122500000</v>
-      </c>
-      <c r="D24" s="31" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="E24" s="32" t="n">
-        <v>17</v>
-      </c>
-      <c r="F24" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="G24" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="32" t="n">
+      <c r="H23" s="34" t="n">
         <v>7</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H24"/>
+  <autoFilter ref="A3:H23"/>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <conditionalFormatting sqref="C4:C23">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00FFFFFF"/>
+        <color rgb="00EBF0FA"/>
+        <color rgb="002E6DA4"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6388,22 +6076,22 @@
     <col width="19" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
     <col width="23" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="29" customWidth="1" min="16" max="16"/>
     <col width="6" customWidth="1" min="17" max="17"/>
     <col width="6" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Appendix D: Impact Projections</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-15</t>
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
         </is>
       </c>
     </row>
@@ -6485,7 +6173,7 @@
       </c>
       <c r="P3" s="14" t="inlineStr">
         <is>
-          <t>Native Area</t>
+          <t>Native Area (CDE-declared)</t>
         </is>
       </c>
       <c r="Q3" s="14" t="inlineStr">
@@ -6525,31 +6213,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F4" s="27" t="n">
+      <c r="F4" s="28" t="n">
         <v>8500000</v>
       </c>
-      <c r="G4" s="27" t="n">
+      <c r="G4" s="28" t="n">
         <v>12500000</v>
       </c>
-      <c r="H4" s="27" t="n">
+      <c r="H4" s="29" t="n">
         <v>52</v>
       </c>
-      <c r="I4" s="27" t="n">
+      <c r="I4" s="29" t="n">
         <v>18</v>
       </c>
-      <c r="J4" s="27" t="n">
+      <c r="J4" s="29" t="n">
         <v>70</v>
       </c>
-      <c r="K4" s="27" t="n">
+      <c r="K4" s="28" t="n">
         <v>240385</v>
       </c>
-      <c r="L4" s="27" t="n">
+      <c r="L4" s="28" t="n">
         <v>163462</v>
       </c>
-      <c r="M4" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="27" t="n">
+      <c r="M4" s="29" t="n">
+        <v/>
+      </c>
+      <c r="N4" s="29" t="n">
         <v>24000</v>
       </c>
       <c r="O4" s="5" t="inlineStr">
@@ -6599,31 +6287,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F5" s="29" t="n">
+      <c r="F5" s="30" t="n">
         <v>7000000</v>
       </c>
-      <c r="G5" s="29" t="n">
+      <c r="G5" s="30" t="n">
         <v>9800000</v>
       </c>
-      <c r="H5" s="29" t="n">
+      <c r="H5" s="31" t="n">
         <v>38</v>
       </c>
-      <c r="I5" s="29" t="n">
+      <c r="I5" s="31" t="n">
         <v>22</v>
       </c>
-      <c r="J5" s="29" t="n">
+      <c r="J5" s="31" t="n">
         <v>60</v>
       </c>
-      <c r="K5" s="29" t="n">
+      <c r="K5" s="30" t="n">
         <v>257895</v>
       </c>
-      <c r="L5" s="29" t="n">
+      <c r="L5" s="30" t="n">
         <v>184211</v>
       </c>
-      <c r="M5" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="29" t="n">
+      <c r="M5" s="31" t="n">
+        <v/>
+      </c>
+      <c r="N5" s="31" t="n">
         <v>0</v>
       </c>
       <c r="O5" s="7" t="inlineStr">
@@ -6673,31 +6361,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="28" t="n">
         <v>5000000</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="28" t="n">
         <v>7200000</v>
       </c>
-      <c r="H6" s="27" t="n">
+      <c r="H6" s="29" t="n">
         <v>65</v>
       </c>
-      <c r="I6" s="27" t="n">
+      <c r="I6" s="29" t="n">
         <v>8</v>
       </c>
-      <c r="J6" s="27" t="n">
+      <c r="J6" s="29" t="n">
         <v>73</v>
       </c>
-      <c r="K6" s="27" t="n">
+      <c r="K6" s="28" t="n">
         <v>110769</v>
       </c>
-      <c r="L6" s="27" t="n">
+      <c r="L6" s="28" t="n">
         <v>76923</v>
       </c>
-      <c r="M6" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="27" t="n">
+      <c r="M6" s="29" t="n">
+        <v/>
+      </c>
+      <c r="N6" s="29" t="n">
         <v>18000</v>
       </c>
       <c r="O6" s="5" t="inlineStr">
@@ -6747,31 +6435,31 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="F7" s="29" t="n">
+      <c r="F7" s="30" t="n">
         <v>4500000</v>
       </c>
-      <c r="G7" s="29" t="n">
+      <c r="G7" s="30" t="n">
         <v>6000000</v>
       </c>
-      <c r="H7" s="29" t="n">
+      <c r="H7" s="31" t="n">
         <v>80</v>
       </c>
-      <c r="I7" s="29" t="n">
+      <c r="I7" s="31" t="n">
         <v>25</v>
       </c>
-      <c r="J7" s="29" t="n">
+      <c r="J7" s="31" t="n">
         <v>105</v>
       </c>
-      <c r="K7" s="29" t="n">
+      <c r="K7" s="30" t="n">
         <v>75000</v>
       </c>
-      <c r="L7" s="29" t="n">
+      <c r="L7" s="30" t="n">
         <v>56250</v>
       </c>
-      <c r="M7" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="29" t="n">
+      <c r="M7" s="31" t="n">
+        <v/>
+      </c>
+      <c r="N7" s="31" t="n">
         <v>0</v>
       </c>
       <c r="O7" s="7" t="inlineStr">
@@ -6821,31 +6509,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="28" t="n">
         <v>7500000</v>
       </c>
-      <c r="G8" s="27" t="n">
+      <c r="G8" s="28" t="n">
         <v>10000000</v>
       </c>
-      <c r="H8" s="27" t="n">
+      <c r="H8" s="29" t="n">
         <v>42</v>
       </c>
-      <c r="I8" s="27" t="n">
+      <c r="I8" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="J8" s="27" t="n">
+      <c r="J8" s="29" t="n">
         <v>72</v>
       </c>
-      <c r="K8" s="27" t="n">
+      <c r="K8" s="28" t="n">
         <v>238095</v>
       </c>
-      <c r="L8" s="27" t="n">
+      <c r="L8" s="28" t="n">
         <v>178571</v>
       </c>
-      <c r="M8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="27" t="n">
+      <c r="M8" s="29" t="n">
+        <v/>
+      </c>
+      <c r="N8" s="29" t="n">
         <v>20000</v>
       </c>
       <c r="O8" s="5" t="inlineStr">
@@ -6895,31 +6583,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F9" s="29" t="n">
+      <c r="F9" s="30" t="n">
         <v>9000000</v>
       </c>
-      <c r="G9" s="29" t="n">
+      <c r="G9" s="30" t="n">
         <v>14000000</v>
       </c>
-      <c r="H9" s="29" t="n">
+      <c r="H9" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="I9" s="29" t="n">
+      <c r="I9" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="J9" s="29" t="n">
+      <c r="J9" s="31" t="n">
         <v>20</v>
       </c>
-      <c r="K9" s="29" t="n">
+      <c r="K9" s="30" t="n">
         <v>933333</v>
       </c>
-      <c r="L9" s="29" t="n">
+      <c r="L9" s="30" t="n">
         <v>600000</v>
       </c>
-      <c r="M9" s="29" t="n">
+      <c r="M9" s="31" t="n">
         <v>72</v>
       </c>
-      <c r="N9" s="29" t="n">
+      <c r="N9" s="31" t="n">
         <v>0</v>
       </c>
       <c r="O9" s="7" t="inlineStr">
@@ -6969,31 +6657,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="28" t="n">
         <v>4000000</v>
       </c>
-      <c r="G10" s="27" t="n">
+      <c r="G10" s="28" t="n">
         <v>5500000</v>
       </c>
-      <c r="H10" s="27" t="n">
+      <c r="H10" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="I10" s="27" t="n">
+      <c r="I10" s="29" t="n">
         <v>10</v>
       </c>
-      <c r="J10" s="27" t="n">
+      <c r="J10" s="29" t="n">
         <v>38</v>
       </c>
-      <c r="K10" s="27" t="n">
+      <c r="K10" s="28" t="n">
         <v>196429</v>
       </c>
-      <c r="L10" s="27" t="n">
+      <c r="L10" s="28" t="n">
         <v>142857</v>
       </c>
-      <c r="M10" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="27" t="n">
+      <c r="M10" s="29" t="n">
+        <v/>
+      </c>
+      <c r="N10" s="29" t="n">
         <v>12000</v>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -7043,31 +6731,31 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="F11" s="29" t="n">
+      <c r="F11" s="30" t="n">
         <v>8000000</v>
       </c>
-      <c r="G11" s="29" t="n">
+      <c r="G11" s="30" t="n">
         <v>11000000</v>
       </c>
-      <c r="H11" s="29" t="n">
+      <c r="H11" s="31" t="n">
         <v>55</v>
       </c>
-      <c r="I11" s="29" t="n">
+      <c r="I11" s="31" t="n">
         <v>20</v>
       </c>
-      <c r="J11" s="29" t="n">
+      <c r="J11" s="31" t="n">
         <v>75</v>
       </c>
-      <c r="K11" s="29" t="n">
+      <c r="K11" s="30" t="n">
         <v>200000</v>
       </c>
-      <c r="L11" s="29" t="n">
+      <c r="L11" s="30" t="n">
         <v>145455</v>
       </c>
-      <c r="M11" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="29" t="n">
+      <c r="M11" s="31" t="n">
+        <v/>
+      </c>
+      <c r="N11" s="31" t="n">
         <v>22000</v>
       </c>
       <c r="O11" s="7" t="inlineStr">
@@ -7117,31 +6805,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="28" t="n">
         <v>6000000</v>
       </c>
-      <c r="G12" s="27" t="n">
+      <c r="G12" s="28" t="n">
         <v>8200000</v>
       </c>
-      <c r="H12" s="27" t="n">
+      <c r="H12" s="29" t="n">
         <v>35</v>
       </c>
-      <c r="I12" s="27" t="n">
+      <c r="I12" s="29" t="n">
         <v>8</v>
       </c>
-      <c r="J12" s="27" t="n">
+      <c r="J12" s="29" t="n">
         <v>43</v>
       </c>
-      <c r="K12" s="27" t="n">
+      <c r="K12" s="28" t="n">
         <v>234286</v>
       </c>
-      <c r="L12" s="27" t="n">
+      <c r="L12" s="28" t="n">
         <v>171429</v>
       </c>
-      <c r="M12" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="27" t="n">
+      <c r="M12" s="29" t="n">
+        <v/>
+      </c>
+      <c r="N12" s="29" t="n">
         <v>16000</v>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -7191,31 +6879,31 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="F13" s="29" t="n">
+      <c r="F13" s="30" t="n">
         <v>3500000</v>
       </c>
-      <c r="G13" s="29" t="n">
+      <c r="G13" s="30" t="n">
         <v>4800000</v>
       </c>
-      <c r="H13" s="29" t="n">
+      <c r="H13" s="31" t="n">
         <v>90</v>
       </c>
-      <c r="I13" s="29" t="n">
+      <c r="I13" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="J13" s="29" t="n">
+      <c r="J13" s="31" t="n">
         <v>105</v>
       </c>
-      <c r="K13" s="29" t="n">
+      <c r="K13" s="30" t="n">
         <v>53333</v>
       </c>
-      <c r="L13" s="29" t="n">
+      <c r="L13" s="30" t="n">
         <v>38889</v>
       </c>
-      <c r="M13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="29" t="n">
+      <c r="M13" s="31" t="n">
+        <v/>
+      </c>
+      <c r="N13" s="31" t="n">
         <v>0</v>
       </c>
       <c r="O13" s="7" t="inlineStr">
@@ -7265,31 +6953,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F14" s="27" t="n">
+      <c r="F14" s="28" t="n">
         <v>9500000</v>
       </c>
-      <c r="G14" s="27" t="n">
+      <c r="G14" s="28" t="n">
         <v>13500000</v>
       </c>
-      <c r="H14" s="27" t="n">
+      <c r="H14" s="29" t="n">
         <v>12</v>
       </c>
-      <c r="I14" s="27" t="n">
+      <c r="I14" s="29" t="n">
         <v>4</v>
       </c>
-      <c r="J14" s="27" t="n">
+      <c r="J14" s="29" t="n">
         <v>16</v>
       </c>
-      <c r="K14" s="27" t="n">
+      <c r="K14" s="28" t="n">
         <v>1125000</v>
       </c>
-      <c r="L14" s="27" t="n">
+      <c r="L14" s="28" t="n">
         <v>791667</v>
       </c>
-      <c r="M14" s="27" t="n">
+      <c r="M14" s="29" t="n">
         <v>64</v>
       </c>
-      <c r="N14" s="27" t="n">
+      <c r="N14" s="29" t="n">
         <v>0</v>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -7339,31 +7027,31 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="F15" s="29" t="n">
+      <c r="F15" s="30" t="n">
         <v>3800000</v>
       </c>
-      <c r="G15" s="29" t="n">
+      <c r="G15" s="30" t="n">
         <v>5000000</v>
       </c>
-      <c r="H15" s="29" t="n">
+      <c r="H15" s="31" t="n">
         <v>22</v>
       </c>
-      <c r="I15" s="29" t="n">
+      <c r="I15" s="31" t="n">
         <v>6</v>
       </c>
-      <c r="J15" s="29" t="n">
+      <c r="J15" s="31" t="n">
         <v>28</v>
       </c>
-      <c r="K15" s="29" t="n">
+      <c r="K15" s="30" t="n">
         <v>227273</v>
       </c>
-      <c r="L15" s="29" t="n">
+      <c r="L15" s="30" t="n">
         <v>172727</v>
       </c>
-      <c r="M15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="29" t="n">
+      <c r="M15" s="31" t="n">
+        <v/>
+      </c>
+      <c r="N15" s="31" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="7" t="inlineStr">
@@ -7413,36 +7101,36 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F16" s="27" t="n">
+      <c r="F16" s="28" t="n">
         <v>5500000</v>
       </c>
-      <c r="G16" s="27" t="n">
+      <c r="G16" s="28" t="n">
         <v>7500000</v>
       </c>
-      <c r="H16" s="27" t="n">
+      <c r="H16" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="I16" s="27" t="n">
+      <c r="I16" s="29" t="n">
         <v>12</v>
       </c>
-      <c r="J16" s="27" t="n">
+      <c r="J16" s="29" t="n">
         <v>42</v>
       </c>
-      <c r="K16" s="27" t="n">
+      <c r="K16" s="28" t="n">
         <v>250000</v>
       </c>
-      <c r="L16" s="27" t="n">
+      <c r="L16" s="28" t="n">
         <v>183333</v>
       </c>
-      <c r="M16" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="27" t="n">
+      <c r="M16" s="29" t="n">
+        <v/>
+      </c>
+      <c r="N16" s="29" t="n">
         <v>14000</v>
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
-          <t>Deep Distress</t>
+          <t>Severely Distressed</t>
         </is>
       </c>
       <c r="P16" s="5" t="inlineStr">
@@ -7487,31 +7175,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F17" s="29" t="n">
+      <c r="F17" s="30" t="n">
         <v>6500000</v>
       </c>
-      <c r="G17" s="29" t="n">
+      <c r="G17" s="30" t="n">
         <v>9000000</v>
       </c>
-      <c r="H17" s="29" t="n">
+      <c r="H17" s="31" t="n">
         <v>48</v>
       </c>
-      <c r="I17" s="29" t="n">
+      <c r="I17" s="31" t="n">
         <v>25</v>
       </c>
-      <c r="J17" s="29" t="n">
+      <c r="J17" s="31" t="n">
         <v>73</v>
       </c>
-      <c r="K17" s="29" t="n">
+      <c r="K17" s="30" t="n">
         <v>187500</v>
       </c>
-      <c r="L17" s="29" t="n">
+      <c r="L17" s="30" t="n">
         <v>135417</v>
       </c>
-      <c r="M17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="29" t="n">
+      <c r="M17" s="31" t="n">
+        <v/>
+      </c>
+      <c r="N17" s="31" t="n">
         <v>18500</v>
       </c>
       <c r="O17" s="7" t="inlineStr">
@@ -7561,31 +7249,31 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="F18" s="27" t="n">
+      <c r="F18" s="28" t="n">
         <v>5000000</v>
       </c>
-      <c r="G18" s="27" t="n">
+      <c r="G18" s="28" t="n">
         <v>6500000</v>
       </c>
-      <c r="H18" s="27" t="n">
+      <c r="H18" s="29" t="n">
         <v>110</v>
       </c>
-      <c r="I18" s="27" t="n">
+      <c r="I18" s="29" t="n">
         <v>45</v>
       </c>
-      <c r="J18" s="27" t="n">
+      <c r="J18" s="29" t="n">
         <v>155</v>
       </c>
-      <c r="K18" s="27" t="n">
+      <c r="K18" s="28" t="n">
         <v>59091</v>
       </c>
-      <c r="L18" s="27" t="n">
+      <c r="L18" s="28" t="n">
         <v>45455</v>
       </c>
-      <c r="M18" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="27" t="n">
+      <c r="M18" s="29" t="n">
+        <v/>
+      </c>
+      <c r="N18" s="29" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="5" t="inlineStr">
@@ -7635,31 +7323,31 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="F19" s="29" t="n">
+      <c r="F19" s="30" t="n">
         <v>7500000</v>
       </c>
-      <c r="G19" s="29" t="n">
+      <c r="G19" s="30" t="n">
         <v>10500000</v>
       </c>
-      <c r="H19" s="29" t="n">
+      <c r="H19" s="31" t="n">
         <v>35</v>
       </c>
-      <c r="I19" s="29" t="n">
+      <c r="I19" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="J19" s="29" t="n">
+      <c r="J19" s="31" t="n">
         <v>45</v>
       </c>
-      <c r="K19" s="29" t="n">
+      <c r="K19" s="30" t="n">
         <v>300000</v>
       </c>
-      <c r="L19" s="29" t="n">
+      <c r="L19" s="30" t="n">
         <v>214286</v>
       </c>
-      <c r="M19" s="29" t="n">
+      <c r="M19" s="31" t="n">
         <v>24</v>
       </c>
-      <c r="N19" s="29" t="n">
+      <c r="N19" s="31" t="n">
         <v>20000</v>
       </c>
       <c r="O19" s="7" t="inlineStr">
@@ -7709,31 +7397,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F20" s="27" t="n">
+      <c r="F20" s="28" t="n">
         <v>3200000</v>
       </c>
-      <c r="G20" s="27" t="n">
+      <c r="G20" s="28" t="n">
         <v>4200000</v>
       </c>
-      <c r="H20" s="27" t="n">
+      <c r="H20" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="I20" s="27" t="n">
+      <c r="I20" s="29" t="n">
         <v>15</v>
       </c>
-      <c r="J20" s="27" t="n">
+      <c r="J20" s="29" t="n">
         <v>35</v>
       </c>
-      <c r="K20" s="27" t="n">
+      <c r="K20" s="28" t="n">
         <v>210000</v>
       </c>
-      <c r="L20" s="27" t="n">
+      <c r="L20" s="28" t="n">
         <v>160000</v>
       </c>
-      <c r="M20" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="27" t="n">
+      <c r="M20" s="29" t="n">
+        <v/>
+      </c>
+      <c r="N20" s="29" t="n">
         <v>8000</v>
       </c>
       <c r="O20" s="5" t="inlineStr">
@@ -7770,7 +7458,7 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>KS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -7783,31 +7471,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F21" s="29" t="n">
+      <c r="F21" s="30" t="n">
         <v>8500000</v>
       </c>
-      <c r="G21" s="29" t="n">
+      <c r="G21" s="30" t="n">
         <v>11800000</v>
       </c>
-      <c r="H21" s="29" t="n">
+      <c r="H21" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="I21" s="29" t="n">
+      <c r="I21" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="J21" s="29" t="n">
+      <c r="J21" s="31" t="n">
         <v>13</v>
       </c>
-      <c r="K21" s="29" t="n">
+      <c r="K21" s="30" t="n">
         <v>1180000</v>
       </c>
-      <c r="L21" s="29" t="n">
+      <c r="L21" s="30" t="n">
         <v>850000</v>
       </c>
-      <c r="M21" s="29" t="n">
+      <c r="M21" s="31" t="n">
         <v>56</v>
       </c>
-      <c r="N21" s="29" t="n">
+      <c r="N21" s="31" t="n">
         <v>0</v>
       </c>
       <c r="O21" s="7" t="inlineStr">
@@ -7857,31 +7545,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F22" s="27" t="n">
+      <c r="F22" s="28" t="n">
         <v>4200000</v>
       </c>
-      <c r="G22" s="27" t="n">
+      <c r="G22" s="28" t="n">
         <v>5800000</v>
       </c>
-      <c r="H22" s="27" t="n">
+      <c r="H22" s="29" t="n">
         <v>45</v>
       </c>
-      <c r="I22" s="27" t="n">
+      <c r="I22" s="29" t="n">
         <v>8</v>
       </c>
-      <c r="J22" s="27" t="n">
+      <c r="J22" s="29" t="n">
         <v>53</v>
       </c>
-      <c r="K22" s="27" t="n">
+      <c r="K22" s="28" t="n">
         <v>128889</v>
       </c>
-      <c r="L22" s="27" t="n">
+      <c r="L22" s="28" t="n">
         <v>93333</v>
       </c>
-      <c r="M22" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="27" t="n">
+      <c r="M22" s="29" t="n">
+        <v/>
+      </c>
+      <c r="N22" s="29" t="n">
         <v>11000</v>
       </c>
       <c r="O22" s="5" t="inlineStr">
@@ -7931,31 +7619,31 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="F23" s="29" t="n">
+      <c r="F23" s="30" t="n">
         <v>5800000</v>
       </c>
-      <c r="G23" s="29" t="n">
+      <c r="G23" s="30" t="n">
         <v>7800000</v>
       </c>
-      <c r="H23" s="29" t="n">
+      <c r="H23" s="31" t="n">
         <v>32</v>
       </c>
-      <c r="I23" s="29" t="n">
+      <c r="I23" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="J23" s="29" t="n">
+      <c r="J23" s="31" t="n">
         <v>41</v>
       </c>
-      <c r="K23" s="29" t="n">
+      <c r="K23" s="30" t="n">
         <v>243750</v>
       </c>
-      <c r="L23" s="29" t="n">
+      <c r="L23" s="30" t="n">
         <v>181250</v>
       </c>
-      <c r="M23" s="29" t="n">
+      <c r="M23" s="31" t="n">
         <v>18</v>
       </c>
-      <c r="N23" s="29" t="n">
+      <c r="N23" s="31" t="n">
         <v>15000</v>
       </c>
       <c r="O23" s="7" t="inlineStr">
@@ -7980,50 +7668,50 @@
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B24" s="31" t="inlineStr">
+      <c r="B24" s="32" t="inlineStr">
         <is>
           <t>20 Projects</t>
         </is>
       </c>
-      <c r="C24" s="31" t="inlineStr"/>
-      <c r="D24" s="31" t="inlineStr"/>
-      <c r="E24" s="31" t="inlineStr"/>
-      <c r="F24" s="32" t="n">
+      <c r="C24" s="32" t="inlineStr"/>
+      <c r="D24" s="32" t="inlineStr"/>
+      <c r="E24" s="32" t="inlineStr"/>
+      <c r="F24" s="33" t="n">
         <v>122500000</v>
       </c>
-      <c r="G24" s="32" t="n">
+      <c r="G24" s="33" t="n">
         <v>170600000</v>
       </c>
-      <c r="H24" s="32" t="n">
+      <c r="H24" s="34" t="n">
         <v>864</v>
       </c>
-      <c r="I24" s="32" t="n">
+      <c r="I24" s="34" t="n">
         <v>298</v>
       </c>
-      <c r="J24" s="32" t="n">
+      <c r="J24" s="34" t="n">
         <v>1162</v>
       </c>
-      <c r="K24" s="32" t="n">
+      <c r="K24" s="33" t="n">
         <v>197454</v>
       </c>
-      <c r="L24" s="32" t="n">
+      <c r="L24" s="33" t="n">
         <v>141782</v>
       </c>
-      <c r="M24" s="32" t="n">
+      <c r="M24" s="34" t="n">
         <v>234</v>
       </c>
-      <c r="N24" s="32" t="n">
+      <c r="N24" s="34" t="n">
         <v>198500</v>
       </c>
-      <c r="O24" s="31" t="inlineStr"/>
-      <c r="P24" s="31" t="inlineStr"/>
-      <c r="Q24" s="31" t="inlineStr"/>
-      <c r="R24" s="31" t="inlineStr"/>
+      <c r="O24" s="32" t="inlineStr"/>
+      <c r="P24" s="32" t="inlineStr"/>
+      <c r="Q24" s="32" t="inlineStr"/>
+      <c r="R24" s="32" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:R24"/>
@@ -8055,16 +7743,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Section D: Investor Commitments</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-15</t>
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
         </is>
       </c>
     </row>
@@ -8195,26 +7883,26 @@
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B6" s="31" t="inlineStr"/>
-      <c r="C6" s="31" t="inlineStr"/>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="B6" s="32" t="inlineStr"/>
+      <c r="C6" s="32" t="inlineStr"/>
+      <c r="D6" s="32" t="inlineStr">
         <is>
           <t>[CDE TO COMPLETE]</t>
         </is>
       </c>
-      <c r="E6" s="31" t="inlineStr"/>
-      <c r="F6" s="31" t="inlineStr"/>
-      <c r="G6" s="31" t="inlineStr">
+      <c r="E6" s="32" t="inlineStr"/>
+      <c r="F6" s="32" t="inlineStr"/>
+      <c r="G6" s="32" t="inlineStr">
         <is>
           <t>[CDE TO COMPLETE: This table is a blank form. nmtc-application-builder holds no investor data for your CDE and supplies no figure in it — not a name, a type, a CRA obligation, a commitment amount, a credit price or a status, and not the number of rows. Add one row per investor you can name and defend to the CDFI Fund, and delete any row you cannot.]</t>
         </is>
       </c>
-      <c r="H6" s="31" t="inlineStr">
+      <c r="H6" s="32" t="inlineStr">
         <is>
           <t>[CDE TO COMPLETE]</t>
         </is>
@@ -8248,16 +7936,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Appendix E: CDE Track Record</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-15</t>
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
         </is>
       </c>
     </row>
@@ -8294,10 +7982,10 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="27" t="n">
+      <c r="A4" s="36" t="n">
         <v>2019</v>
       </c>
-      <c r="B4" s="27" t="n">
+      <c r="B4" s="28" t="n">
         <v>40000000</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -8318,10 +8006,10 @@
       <c r="F4" s="5" t="inlineStr"/>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="29" t="n">
+      <c r="A5" s="37" t="n">
         <v>2021</v>
       </c>
-      <c r="B5" s="29" t="n">
+      <c r="B5" s="30" t="n">
         <v>55000000</v>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -8342,10 +8030,10 @@
       <c r="F5" s="7" t="inlineStr"/>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="27" t="n">
+      <c r="A6" s="36" t="n">
         <v>2023</v>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="28" t="n">
         <v>60000000</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -8366,26 +8054,26 @@
       <c r="F6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="31" t="inlineStr">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B7" s="32" t="n">
+      <c r="B7" s="33" t="n">
         <v>155000000</v>
       </c>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="32" t="inlineStr">
         <is>
           <t>2 rounds fully deployed</t>
         </is>
       </c>
-      <c r="D7" s="31" t="inlineStr">
+      <c r="D7" s="32" t="inlineStr">
         <is>
           <t>7 states</t>
         </is>
       </c>
-      <c r="E7" s="31" t="inlineStr"/>
-      <c r="F7" s="31" t="inlineStr">
+      <c r="E7" s="32" t="inlineStr"/>
+      <c r="F7" s="32" t="inlineStr">
         <is>
           <t>$155,000,000 total prior allocation</t>
         </is>

</xml_diff>

<commit_message>
Deployed 63443cc with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -874,7 +874,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>CY2025  |  Prepared: August 16, 2026  |  Readiness Grade: A (86.6/100)</t>
+          <t>CY2025  |  Prepared: August 17, 2026  |  Readiness Grade: A (86.6/100)</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-16</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="27" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3727,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="27" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
         </is>
       </c>
     </row>
@@ -5424,7 +5424,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="27" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
         </is>
       </c>
     </row>
@@ -6091,7 +6091,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="27" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
         </is>
       </c>
     </row>
@@ -7752,7 +7752,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="27" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
         </is>
       </c>
     </row>
@@ -7945,7 +7945,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="27" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 0643296 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -8,20 +8,21 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Detail" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distress Documentation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geographic Targeting" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Projections" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investor Commitments" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track Record" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q25 Basis Note" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distress Documentation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geographic Targeting" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Projections" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investor Commitments" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track Record" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipeline Detail'!$A$3:$AC$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Distress Documentation'!$A$3:$O$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Geographic Targeting'!$A$3:$H$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Impact Projections'!$A$3:$R$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Investor Commitments'!$A$3:$H$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Track Record'!$A$3:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pipeline Detail'!$A$3:$AC$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Distress Documentation'!$A$3:$O$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Geographic Targeting'!$A$3:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Impact Projections'!$A$3:$R$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Investor Commitments'!$A$3:$H$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Track Record'!$A$3:$F$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -34,7 +35,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -106,6 +107,16 @@
       <i val="1"/>
       <color rgb="006B6B6B"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="006B6B6B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A1A1A"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -223,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -296,7 +307,16 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -874,7 +894,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>CY2025  |  Prepared: August 17, 2026  |  Readiness Grade: A (86.6/100)</t>
+          <t>CY2025  |  Prepared: August 19, 2026  |  Readiness Grade: A (86.6/100)</t>
         </is>
       </c>
     </row>
@@ -885,7 +905,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1">
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Total NMTC Allocation Requested</t>
@@ -895,7 +915,7 @@
         <v>65000000</v>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1">
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Total QEI in Pipeline</t>
@@ -905,7 +925,7 @@
         <v>122500000</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Total Project Cost</t>
@@ -915,7 +935,7 @@
         <v>170600000</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Number of Projects</t>
@@ -925,7 +945,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>States Represented</t>
@@ -935,7 +955,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>NMTC Eligibility Rate</t>
@@ -945,17 +965,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
+    <row r="12" ht="45" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Deep/Severe Distress Concentration</t>
+          <t>Deep/Severe Distress Concentration (a share of QEI, not of QLICIs — see the 'Q25 Basis Note' sheet)</t>
         </is>
       </c>
       <c r="C12" s="12" t="n">
         <v>0.866938775510204</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13" ht="15" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Total Jobs to Be Created</t>
@@ -965,7 +985,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
+    <row r="14" ht="15" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Jobs per $1MM QEI</t>
@@ -1093,7 +1113,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="36" customHeight="1">
       <c r="A25" s="24" t="inlineStr">
         <is>
           <t>READINESS SCORE BREAKDOWN — weights are this tool's own unsourced judgement (eligibility quality 25%; distress concentration 25%; geographic diversity 15%; impact metrics 20%; validation pass rate 10%; completeness 5%); the CDFI Fund publishes no such weighting and this score does not predict an award outcome.</t>
@@ -1103,7 +1123,7 @@
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-17</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-19</t>
         </is>
       </c>
     </row>
@@ -1154,6 +1174,94 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>BASIS NOTE — the CDFI Fund's two distress commitments are measured on QLICIs, not on QEI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>This note is the basis for 'Deep/Severe Distress Concentration' on the Summary Dashboard, and for the Deep Distress and Severely Distressed rows of Section B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="84" customHeight="1">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Question 25 of the CY 2024-2025 NMTC Allocation Application (printed pp. 38-41) sets both commitments, and both are measured on QLICIs — specifically on QLICIs "in terms of aggregate dollar amounts", tested for each QLICI. Question 25(a) asks for at least 85% of QLICIs in areas characterized by at least ONE of items 1-5 (Severe Distress; NMTC Native Areas; U.S. Island Areas; Non-Metropolitan Counties; Targeted Populations) or by at least TWO of items 6-12 (25% poverty / 70% median family income / 1.25x unemployment; Brownfield Sites; ARC and/or DRA Areas; Colonias Areas; Federal Medically Underserved Areas; FEMA Disaster Areas; Low-Income and Low-Access to Supermarkets).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="98" customHeight="1">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>"Multiple indicia of distress" is that two-of-seven test, applied per QLICI — not a loose notion of compounded distress and not a category of its own. Question 25(b)(i) is NOT a 20% bar. It is a selectable commitment level — 0, 5, 10, 15 or 20, and selecting 20 opens a field for any figure from 20% to 100% — over FOUR qualifying area types: Deep Distress, NMTC Native Areas, High Migration Rural Counties and U.S. Island Areas. A CDE that can honestly commit 10% selects 10 and has failed nothing; a CDE whose QLICIs sit in Native Areas, High Migration Rural Counties or Island Areas must count them, and no Deep Distress figure in this document does. The Application further states that "A QLICI that meets this commitment will also automatically meet the commitment made in Question 25(a)."</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Every distress share in this document is a share of QEI. nmtc-application-builder computes neither QLICI-denominated figure — it reads this pipeline's QLICI amounts only to print them in Appendix A and to check that each is no larger than its QEI — so no figure in this document answers either commitment, and none may be presented to the CDFI Fund as doing so. WHICH OF THE CDE'S QUALIFYING ROUTES ARE VISIBLE HERE: this package carries a per-project field for 5 of the 14 distinct area types Question 25 lists, and they do NOT share one provenance, so each is stated with its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="70" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Severe Distress and Deep Distress: TOOL-VERIFIED — the distress level is read from the CDFI Fund eligibility table for the tract this package geocoded, and a CDE's own distress column is kept separately and labelled CDE-declared wherever it is shown. High Migration Rural Counties: CDE-DECLARED AND TOOL-VERIFIED — enrichment overwrites the CDE's declaration whenever nmtc-mapper returns a determination for the tract, so the declaration stands only where the tool reached none, and where enrichment did not run at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="98" customHeight="1">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>NMTC Native Areas and U.S. territory: CDE-DECLARED AND TOOL-UNVERIFIED — nothing in this package checks either one, and a Native Area determination is a spatial intersection against the Fund's CIMS map rather than a tract-keyed lookup this package could perform (U.S. territory is the CDE's own word; the Application's U.S. Island Areas is a specific list of five). It carries NOTHING for Non-Metropolitan Counties, nothing for Targeted Populations, and nothing for any of items 6-12; it computes no multi-indicia measure at all. Holding those fields is not a partial answer to Question 25 and must not be read as one: the commitment is a share of QLICI DOLLARS, this package weights nothing by QLICI dollars, and a flag that enters no denominator contributes nothing to a share.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>Deep Distress is a strict subset of severe distress, so the severe-distress share already includes the deep-distress share. The CDE must compute both QLICI-denominated shares from its own QLICI amounts, against the Application's own area lists, before stating either commitment. (The CY 2026 NOAA is not yet published.)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A7:F7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AW24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1189,16 +1297,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Appendix A: Pipeline Detail</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
         </is>
       </c>
     </row>
@@ -1421,25 +1529,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P4" s="28" t="n">
+      <c r="P4" s="31" t="n">
         <v>12500000</v>
       </c>
-      <c r="Q4" s="28" t="n">
+      <c r="Q4" s="31" t="n">
         <v>8500000</v>
       </c>
-      <c r="R4" s="28" t="n">
+      <c r="R4" s="31" t="n">
         <v>8500000</v>
       </c>
-      <c r="S4" s="28" t="n">
+      <c r="S4" s="31" t="n">
         <v>5748550</v>
       </c>
-      <c r="T4" s="28" t="n">
+      <c r="T4" s="31" t="n">
         <v>3315000</v>
       </c>
-      <c r="U4" s="28" t="n">
+      <c r="U4" s="31" t="n">
         <v>2751450</v>
       </c>
-      <c r="V4" s="28" t="n">
+      <c r="V4" s="31" t="n">
         <v>212500</v>
       </c>
       <c r="W4" s="5" t="inlineStr"/>
@@ -1449,16 +1557,16 @@
           <t>2025-09-30</t>
         </is>
       </c>
-      <c r="Z4" s="29" t="n">
+      <c r="Z4" s="32" t="n">
         <v>52</v>
       </c>
-      <c r="AA4" s="29" t="n">
+      <c r="AA4" s="32" t="n">
         <v>18</v>
       </c>
-      <c r="AB4" s="29" t="n">
+      <c r="AB4" s="32" t="n">
         <v/>
       </c>
-      <c r="AC4" s="29" t="n">
+      <c r="AC4" s="32" t="n">
         <v>24000</v>
       </c>
     </row>
@@ -1534,25 +1642,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P5" s="30" t="n">
+      <c r="P5" s="33" t="n">
         <v>9800000</v>
       </c>
-      <c r="Q5" s="30" t="n">
+      <c r="Q5" s="33" t="n">
         <v>7000000</v>
       </c>
-      <c r="R5" s="30" t="n">
+      <c r="R5" s="33" t="n">
         <v>7000000</v>
       </c>
-      <c r="S5" s="30" t="n">
+      <c r="S5" s="33" t="n">
         <v>4734100</v>
       </c>
-      <c r="T5" s="30" t="n">
+      <c r="T5" s="33" t="n">
         <v>2730000</v>
       </c>
-      <c r="U5" s="30" t="n">
+      <c r="U5" s="33" t="n">
         <v>2265900</v>
       </c>
-      <c r="V5" s="30" t="n">
+      <c r="V5" s="33" t="n">
         <v>175000</v>
       </c>
       <c r="W5" s="7" t="inlineStr"/>
@@ -1562,16 +1670,16 @@
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="Z5" s="31" t="n">
+      <c r="Z5" s="34" t="n">
         <v>38</v>
       </c>
-      <c r="AA5" s="31" t="n">
+      <c r="AA5" s="34" t="n">
         <v>22</v>
       </c>
-      <c r="AB5" s="31" t="n">
+      <c r="AB5" s="34" t="n">
         <v/>
       </c>
-      <c r="AC5" s="31" t="n">
+      <c r="AC5" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1647,25 +1755,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P6" s="28" t="n">
+      <c r="P6" s="31" t="n">
         <v>7200000</v>
       </c>
-      <c r="Q6" s="28" t="n">
+      <c r="Q6" s="31" t="n">
         <v>5000000</v>
       </c>
-      <c r="R6" s="28" t="n">
+      <c r="R6" s="31" t="n">
         <v>5000000</v>
       </c>
-      <c r="S6" s="28" t="n">
+      <c r="S6" s="31" t="n">
         <v>3381500</v>
       </c>
-      <c r="T6" s="28" t="n">
+      <c r="T6" s="31" t="n">
         <v>1950000</v>
       </c>
-      <c r="U6" s="28" t="n">
+      <c r="U6" s="31" t="n">
         <v>1618500</v>
       </c>
-      <c r="V6" s="28" t="n">
+      <c r="V6" s="31" t="n">
         <v>125000</v>
       </c>
       <c r="W6" s="5" t="inlineStr"/>
@@ -1675,16 +1783,16 @@
           <t>2025-08-31</t>
         </is>
       </c>
-      <c r="Z6" s="29" t="n">
+      <c r="Z6" s="32" t="n">
         <v>65</v>
       </c>
-      <c r="AA6" s="29" t="n">
+      <c r="AA6" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="AB6" s="29" t="n">
+      <c r="AB6" s="32" t="n">
         <v/>
       </c>
-      <c r="AC6" s="29" t="n">
+      <c r="AC6" s="32" t="n">
         <v>18000</v>
       </c>
     </row>
@@ -1760,25 +1868,25 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="P7" s="30" t="n">
+      <c r="P7" s="33" t="n">
         <v>6000000</v>
       </c>
-      <c r="Q7" s="30" t="n">
+      <c r="Q7" s="33" t="n">
         <v>4500000</v>
       </c>
-      <c r="R7" s="30" t="n">
+      <c r="R7" s="33" t="n">
         <v>4500000</v>
       </c>
-      <c r="S7" s="30" t="n">
+      <c r="S7" s="33" t="n">
         <v>3043350</v>
       </c>
-      <c r="T7" s="30" t="n">
+      <c r="T7" s="33" t="n">
         <v>1755000</v>
       </c>
-      <c r="U7" s="30" t="n">
+      <c r="U7" s="33" t="n">
         <v>1456650</v>
       </c>
-      <c r="V7" s="30" t="n">
+      <c r="V7" s="33" t="n">
         <v>112500</v>
       </c>
       <c r="W7" s="7" t="inlineStr"/>
@@ -1788,16 +1896,16 @@
           <t>2025-11-30</t>
         </is>
       </c>
-      <c r="Z7" s="31" t="n">
+      <c r="Z7" s="34" t="n">
         <v>80</v>
       </c>
-      <c r="AA7" s="31" t="n">
+      <c r="AA7" s="34" t="n">
         <v>25</v>
       </c>
-      <c r="AB7" s="31" t="n">
+      <c r="AB7" s="34" t="n">
         <v/>
       </c>
-      <c r="AC7" s="31" t="n">
+      <c r="AC7" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1873,25 +1981,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P8" s="28" t="n">
+      <c r="P8" s="31" t="n">
         <v>10000000</v>
       </c>
-      <c r="Q8" s="28" t="n">
+      <c r="Q8" s="31" t="n">
         <v>7500000</v>
       </c>
-      <c r="R8" s="28" t="n">
+      <c r="R8" s="31" t="n">
         <v>7500000</v>
       </c>
-      <c r="S8" s="28" t="n">
+      <c r="S8" s="31" t="n">
         <v>5072250</v>
       </c>
-      <c r="T8" s="28" t="n">
+      <c r="T8" s="31" t="n">
         <v>2925000</v>
       </c>
-      <c r="U8" s="28" t="n">
+      <c r="U8" s="31" t="n">
         <v>2427750</v>
       </c>
-      <c r="V8" s="28" t="n">
+      <c r="V8" s="31" t="n">
         <v>187500</v>
       </c>
       <c r="W8" s="5" t="inlineStr"/>
@@ -1901,16 +2009,16 @@
           <t>2026-01-31</t>
         </is>
       </c>
-      <c r="Z8" s="29" t="n">
+      <c r="Z8" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="AA8" s="29" t="n">
+      <c r="AA8" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="AB8" s="29" t="n">
+      <c r="AB8" s="32" t="n">
         <v/>
       </c>
-      <c r="AC8" s="29" t="n">
+      <c r="AC8" s="32" t="n">
         <v>20000</v>
       </c>
     </row>
@@ -1986,25 +2094,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P9" s="30" t="n">
+      <c r="P9" s="33" t="n">
         <v>14000000</v>
       </c>
-      <c r="Q9" s="30" t="n">
+      <c r="Q9" s="33" t="n">
         <v>9000000</v>
       </c>
-      <c r="R9" s="30" t="n">
+      <c r="R9" s="33" t="n">
         <v>9000000</v>
       </c>
-      <c r="S9" s="30" t="n">
+      <c r="S9" s="33" t="n">
         <v>6086700</v>
       </c>
-      <c r="T9" s="30" t="n">
+      <c r="T9" s="33" t="n">
         <v>3510000</v>
       </c>
-      <c r="U9" s="30" t="n">
+      <c r="U9" s="33" t="n">
         <v>2913300</v>
       </c>
-      <c r="V9" s="30" t="n">
+      <c r="V9" s="33" t="n">
         <v>225000</v>
       </c>
       <c r="W9" s="7" t="inlineStr"/>
@@ -2014,16 +2122,16 @@
           <t>2025-10-31</t>
         </is>
       </c>
-      <c r="Z9" s="31" t="n">
+      <c r="Z9" s="34" t="n">
         <v>15</v>
       </c>
-      <c r="AA9" s="31" t="n">
+      <c r="AA9" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="AB9" s="31" t="n">
+      <c r="AB9" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="AC9" s="31" t="n">
+      <c r="AC9" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2099,25 +2207,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P10" s="28" t="n">
+      <c r="P10" s="31" t="n">
         <v>5500000</v>
       </c>
-      <c r="Q10" s="28" t="n">
+      <c r="Q10" s="31" t="n">
         <v>4000000</v>
       </c>
-      <c r="R10" s="28" t="n">
+      <c r="R10" s="31" t="n">
         <v>4000000</v>
       </c>
-      <c r="S10" s="28" t="n">
+      <c r="S10" s="31" t="n">
         <v>2705200</v>
       </c>
-      <c r="T10" s="28" t="n">
+      <c r="T10" s="31" t="n">
         <v>1560000</v>
       </c>
-      <c r="U10" s="28" t="n">
+      <c r="U10" s="31" t="n">
         <v>1294800</v>
       </c>
-      <c r="V10" s="28" t="n">
+      <c r="V10" s="31" t="n">
         <v>100000</v>
       </c>
       <c r="W10" s="5" t="inlineStr"/>
@@ -2127,16 +2235,16 @@
           <t>2025-09-15</t>
         </is>
       </c>
-      <c r="Z10" s="29" t="n">
+      <c r="Z10" s="32" t="n">
         <v>28</v>
       </c>
-      <c r="AA10" s="29" t="n">
+      <c r="AA10" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="AB10" s="29" t="n">
+      <c r="AB10" s="32" t="n">
         <v/>
       </c>
-      <c r="AC10" s="29" t="n">
+      <c r="AC10" s="32" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -2212,25 +2320,25 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="P11" s="30" t="n">
+      <c r="P11" s="33" t="n">
         <v>11000000</v>
       </c>
-      <c r="Q11" s="30" t="n">
+      <c r="Q11" s="33" t="n">
         <v>8000000</v>
       </c>
-      <c r="R11" s="30" t="n">
+      <c r="R11" s="33" t="n">
         <v>8000000</v>
       </c>
-      <c r="S11" s="30" t="n">
+      <c r="S11" s="33" t="n">
         <v>5410400</v>
       </c>
-      <c r="T11" s="30" t="n">
+      <c r="T11" s="33" t="n">
         <v>3120000</v>
       </c>
-      <c r="U11" s="30" t="n">
+      <c r="U11" s="33" t="n">
         <v>2589600</v>
       </c>
-      <c r="V11" s="30" t="n">
+      <c r="V11" s="33" t="n">
         <v>200000</v>
       </c>
       <c r="W11" s="7" t="inlineStr"/>
@@ -2240,16 +2348,16 @@
           <t>2026-03-31</t>
         </is>
       </c>
-      <c r="Z11" s="31" t="n">
+      <c r="Z11" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="AA11" s="31" t="n">
+      <c r="AA11" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="AB11" s="31" t="n">
+      <c r="AB11" s="34" t="n">
         <v/>
       </c>
-      <c r="AC11" s="31" t="n">
+      <c r="AC11" s="34" t="n">
         <v>22000</v>
       </c>
     </row>
@@ -2325,25 +2433,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P12" s="28" t="n">
+      <c r="P12" s="31" t="n">
         <v>8200000</v>
       </c>
-      <c r="Q12" s="28" t="n">
+      <c r="Q12" s="31" t="n">
         <v>6000000</v>
       </c>
-      <c r="R12" s="28" t="n">
+      <c r="R12" s="31" t="n">
         <v>6000000</v>
       </c>
-      <c r="S12" s="28" t="n">
+      <c r="S12" s="31" t="n">
         <v>4057800</v>
       </c>
-      <c r="T12" s="28" t="n">
+      <c r="T12" s="31" t="n">
         <v>2340000</v>
       </c>
-      <c r="U12" s="28" t="n">
+      <c r="U12" s="31" t="n">
         <v>1942200</v>
       </c>
-      <c r="V12" s="28" t="n">
+      <c r="V12" s="31" t="n">
         <v>150000</v>
       </c>
       <c r="W12" s="5" t="inlineStr"/>
@@ -2353,16 +2461,16 @@
           <t>2025-11-15</t>
         </is>
       </c>
-      <c r="Z12" s="29" t="n">
+      <c r="Z12" s="32" t="n">
         <v>35</v>
       </c>
-      <c r="AA12" s="29" t="n">
+      <c r="AA12" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="AB12" s="29" t="n">
+      <c r="AB12" s="32" t="n">
         <v/>
       </c>
-      <c r="AC12" s="29" t="n">
+      <c r="AC12" s="32" t="n">
         <v>16000</v>
       </c>
     </row>
@@ -2438,25 +2546,25 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="P13" s="30" t="n">
+      <c r="P13" s="33" t="n">
         <v>4800000</v>
       </c>
-      <c r="Q13" s="30" t="n">
+      <c r="Q13" s="33" t="n">
         <v>3500000</v>
       </c>
-      <c r="R13" s="30" t="n">
+      <c r="R13" s="33" t="n">
         <v>3500000</v>
       </c>
-      <c r="S13" s="30" t="n">
+      <c r="S13" s="33" t="n">
         <v>2367050</v>
       </c>
-      <c r="T13" s="30" t="n">
+      <c r="T13" s="33" t="n">
         <v>1365000</v>
       </c>
-      <c r="U13" s="30" t="n">
+      <c r="U13" s="33" t="n">
         <v>1132950</v>
       </c>
-      <c r="V13" s="30" t="n">
+      <c r="V13" s="33" t="n">
         <v>87500</v>
       </c>
       <c r="W13" s="7" t="inlineStr"/>
@@ -2466,16 +2574,16 @@
           <t>2025-08-15</t>
         </is>
       </c>
-      <c r="Z13" s="31" t="n">
+      <c r="Z13" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="AA13" s="31" t="n">
+      <c r="AA13" s="34" t="n">
         <v>15</v>
       </c>
-      <c r="AB13" s="31" t="n">
+      <c r="AB13" s="34" t="n">
         <v/>
       </c>
-      <c r="AC13" s="31" t="n">
+      <c r="AC13" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2551,25 +2659,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P14" s="28" t="n">
+      <c r="P14" s="31" t="n">
         <v>13500000</v>
       </c>
-      <c r="Q14" s="28" t="n">
+      <c r="Q14" s="31" t="n">
         <v>9500000</v>
       </c>
-      <c r="R14" s="28" t="n">
+      <c r="R14" s="31" t="n">
         <v>9500000</v>
       </c>
-      <c r="S14" s="28" t="n">
+      <c r="S14" s="31" t="n">
         <v>6424850</v>
       </c>
-      <c r="T14" s="28" t="n">
+      <c r="T14" s="31" t="n">
         <v>3705000</v>
       </c>
-      <c r="U14" s="28" t="n">
+      <c r="U14" s="31" t="n">
         <v>3075150</v>
       </c>
-      <c r="V14" s="28" t="n">
+      <c r="V14" s="31" t="n">
         <v>237500</v>
       </c>
       <c r="W14" s="5" t="inlineStr"/>
@@ -2579,16 +2687,16 @@
           <t>2026-02-28</t>
         </is>
       </c>
-      <c r="Z14" s="29" t="n">
+      <c r="Z14" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="AA14" s="29" t="n">
+      <c r="AA14" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="AB14" s="29" t="n">
+      <c r="AB14" s="32" t="n">
         <v>64</v>
       </c>
-      <c r="AC14" s="29" t="n">
+      <c r="AC14" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2664,25 +2772,25 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="P15" s="30" t="n">
+      <c r="P15" s="33" t="n">
         <v>5000000</v>
       </c>
-      <c r="Q15" s="30" t="n">
+      <c r="Q15" s="33" t="n">
         <v>3800000</v>
       </c>
-      <c r="R15" s="30" t="n">
+      <c r="R15" s="33" t="n">
         <v>3800000</v>
       </c>
-      <c r="S15" s="30" t="n">
+      <c r="S15" s="33" t="n">
         <v>2569940</v>
       </c>
-      <c r="T15" s="30" t="n">
+      <c r="T15" s="33" t="n">
         <v>1482000</v>
       </c>
-      <c r="U15" s="30" t="n">
+      <c r="U15" s="33" t="n">
         <v>1230060</v>
       </c>
-      <c r="V15" s="30" t="n">
+      <c r="V15" s="33" t="n">
         <v>95000</v>
       </c>
       <c r="W15" s="7" t="inlineStr"/>
@@ -2692,16 +2800,16 @@
           <t>2025-10-15</t>
         </is>
       </c>
-      <c r="Z15" s="31" t="n">
+      <c r="Z15" s="34" t="n">
         <v>22</v>
       </c>
-      <c r="AA15" s="31" t="n">
+      <c r="AA15" s="34" t="n">
         <v>6</v>
       </c>
-      <c r="AB15" s="31" t="n">
+      <c r="AB15" s="34" t="n">
         <v/>
       </c>
-      <c r="AC15" s="31" t="n">
+      <c r="AC15" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2777,25 +2885,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P16" s="28" t="n">
+      <c r="P16" s="31" t="n">
         <v>7500000</v>
       </c>
-      <c r="Q16" s="28" t="n">
+      <c r="Q16" s="31" t="n">
         <v>5500000</v>
       </c>
-      <c r="R16" s="28" t="n">
+      <c r="R16" s="31" t="n">
         <v>5500000</v>
       </c>
-      <c r="S16" s="28" t="n">
+      <c r="S16" s="31" t="n">
         <v>3719650</v>
       </c>
-      <c r="T16" s="28" t="n">
+      <c r="T16" s="31" t="n">
         <v>2145000</v>
       </c>
-      <c r="U16" s="28" t="n">
+      <c r="U16" s="31" t="n">
         <v>1780350</v>
       </c>
-      <c r="V16" s="28" t="n">
+      <c r="V16" s="31" t="n">
         <v>137500</v>
       </c>
       <c r="W16" s="5" t="inlineStr"/>
@@ -2805,16 +2913,16 @@
           <t>2025-12-31</t>
         </is>
       </c>
-      <c r="Z16" s="29" t="n">
+      <c r="Z16" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="AA16" s="29" t="n">
+      <c r="AA16" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="AB16" s="29" t="n">
+      <c r="AB16" s="32" t="n">
         <v/>
       </c>
-      <c r="AC16" s="29" t="n">
+      <c r="AC16" s="32" t="n">
         <v>14000</v>
       </c>
     </row>
@@ -2890,25 +2998,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P17" s="30" t="n">
+      <c r="P17" s="33" t="n">
         <v>9000000</v>
       </c>
-      <c r="Q17" s="30" t="n">
+      <c r="Q17" s="33" t="n">
         <v>6500000</v>
       </c>
-      <c r="R17" s="30" t="n">
+      <c r="R17" s="33" t="n">
         <v>6500000</v>
       </c>
-      <c r="S17" s="30" t="n">
+      <c r="S17" s="33" t="n">
         <v>4395950</v>
       </c>
-      <c r="T17" s="30" t="n">
+      <c r="T17" s="33" t="n">
         <v>2535000</v>
       </c>
-      <c r="U17" s="30" t="n">
+      <c r="U17" s="33" t="n">
         <v>2104050</v>
       </c>
-      <c r="V17" s="30" t="n">
+      <c r="V17" s="33" t="n">
         <v>162500</v>
       </c>
       <c r="W17" s="7" t="inlineStr"/>
@@ -2918,16 +3026,16 @@
           <t>2026-01-15</t>
         </is>
       </c>
-      <c r="Z17" s="31" t="n">
+      <c r="Z17" s="34" t="n">
         <v>48</v>
       </c>
-      <c r="AA17" s="31" t="n">
+      <c r="AA17" s="34" t="n">
         <v>25</v>
       </c>
-      <c r="AB17" s="31" t="n">
+      <c r="AB17" s="34" t="n">
         <v/>
       </c>
-      <c r="AC17" s="31" t="n">
+      <c r="AC17" s="34" t="n">
         <v>18500</v>
       </c>
     </row>
@@ -3003,25 +3111,25 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="P18" s="28" t="n">
+      <c r="P18" s="31" t="n">
         <v>6500000</v>
       </c>
-      <c r="Q18" s="28" t="n">
+      <c r="Q18" s="31" t="n">
         <v>5000000</v>
       </c>
-      <c r="R18" s="28" t="n">
+      <c r="R18" s="31" t="n">
         <v>5000000</v>
       </c>
-      <c r="S18" s="28" t="n">
+      <c r="S18" s="31" t="n">
         <v>3381500</v>
       </c>
-      <c r="T18" s="28" t="n">
+      <c r="T18" s="31" t="n">
         <v>1950000</v>
       </c>
-      <c r="U18" s="28" t="n">
+      <c r="U18" s="31" t="n">
         <v>1618500</v>
       </c>
-      <c r="V18" s="28" t="n">
+      <c r="V18" s="31" t="n">
         <v>125000</v>
       </c>
       <c r="W18" s="5" t="inlineStr"/>
@@ -3031,16 +3139,16 @@
           <t>2025-09-30</t>
         </is>
       </c>
-      <c r="Z18" s="29" t="n">
+      <c r="Z18" s="32" t="n">
         <v>110</v>
       </c>
-      <c r="AA18" s="29" t="n">
+      <c r="AA18" s="32" t="n">
         <v>45</v>
       </c>
-      <c r="AB18" s="29" t="n">
+      <c r="AB18" s="32" t="n">
         <v/>
       </c>
-      <c r="AC18" s="29" t="n">
+      <c r="AC18" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3116,25 +3224,25 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="P19" s="30" t="n">
+      <c r="P19" s="33" t="n">
         <v>10500000</v>
       </c>
-      <c r="Q19" s="30" t="n">
+      <c r="Q19" s="33" t="n">
         <v>7500000</v>
       </c>
-      <c r="R19" s="30" t="n">
+      <c r="R19" s="33" t="n">
         <v>7500000</v>
       </c>
-      <c r="S19" s="30" t="n">
+      <c r="S19" s="33" t="n">
         <v>5072250</v>
       </c>
-      <c r="T19" s="30" t="n">
+      <c r="T19" s="33" t="n">
         <v>2925000</v>
       </c>
-      <c r="U19" s="30" t="n">
+      <c r="U19" s="33" t="n">
         <v>2427750</v>
       </c>
-      <c r="V19" s="30" t="n">
+      <c r="V19" s="33" t="n">
         <v>187500</v>
       </c>
       <c r="W19" s="7" t="inlineStr"/>
@@ -3144,16 +3252,16 @@
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="Z19" s="31" t="n">
+      <c r="Z19" s="34" t="n">
         <v>35</v>
       </c>
-      <c r="AA19" s="31" t="n">
+      <c r="AA19" s="34" t="n">
         <v>10</v>
       </c>
-      <c r="AB19" s="31" t="n">
+      <c r="AB19" s="34" t="n">
         <v>24</v>
       </c>
-      <c r="AC19" s="31" t="n">
+      <c r="AC19" s="34" t="n">
         <v>20000</v>
       </c>
     </row>
@@ -3229,25 +3337,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P20" s="28" t="n">
+      <c r="P20" s="31" t="n">
         <v>4200000</v>
       </c>
-      <c r="Q20" s="28" t="n">
+      <c r="Q20" s="31" t="n">
         <v>3200000</v>
       </c>
-      <c r="R20" s="28" t="n">
+      <c r="R20" s="31" t="n">
         <v>3200000</v>
       </c>
-      <c r="S20" s="28" t="n">
+      <c r="S20" s="31" t="n">
         <v>2164160</v>
       </c>
-      <c r="T20" s="28" t="n">
+      <c r="T20" s="31" t="n">
         <v>1248000</v>
       </c>
-      <c r="U20" s="28" t="n">
+      <c r="U20" s="31" t="n">
         <v>1035840</v>
       </c>
-      <c r="V20" s="28" t="n">
+      <c r="V20" s="31" t="n">
         <v>80000</v>
       </c>
       <c r="W20" s="5" t="inlineStr"/>
@@ -3257,16 +3365,16 @@
           <t>2025-11-30</t>
         </is>
       </c>
-      <c r="Z20" s="29" t="n">
+      <c r="Z20" s="32" t="n">
         <v>20</v>
       </c>
-      <c r="AA20" s="29" t="n">
+      <c r="AA20" s="32" t="n">
         <v>15</v>
       </c>
-      <c r="AB20" s="29" t="n">
+      <c r="AB20" s="32" t="n">
         <v/>
       </c>
-      <c r="AC20" s="29" t="n">
+      <c r="AC20" s="32" t="n">
         <v>8000</v>
       </c>
     </row>
@@ -3342,25 +3450,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P21" s="30" t="n">
+      <c r="P21" s="33" t="n">
         <v>11800000</v>
       </c>
-      <c r="Q21" s="30" t="n">
+      <c r="Q21" s="33" t="n">
         <v>8500000</v>
       </c>
-      <c r="R21" s="30" t="n">
+      <c r="R21" s="33" t="n">
         <v>8500000</v>
       </c>
-      <c r="S21" s="30" t="n">
+      <c r="S21" s="33" t="n">
         <v>5748550</v>
       </c>
-      <c r="T21" s="30" t="n">
+      <c r="T21" s="33" t="n">
         <v>3315000</v>
       </c>
-      <c r="U21" s="30" t="n">
+      <c r="U21" s="33" t="n">
         <v>2751450</v>
       </c>
-      <c r="V21" s="30" t="n">
+      <c r="V21" s="33" t="n">
         <v>212500</v>
       </c>
       <c r="W21" s="7" t="inlineStr"/>
@@ -3370,16 +3478,16 @@
           <t>2026-02-15</t>
         </is>
       </c>
-      <c r="Z21" s="31" t="n">
+      <c r="Z21" s="34" t="n">
         <v>10</v>
       </c>
-      <c r="AA21" s="31" t="n">
+      <c r="AA21" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="AB21" s="31" t="n">
+      <c r="AB21" s="34" t="n">
         <v>56</v>
       </c>
-      <c r="AC21" s="31" t="n">
+      <c r="AC21" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3455,25 +3563,25 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="P22" s="28" t="n">
+      <c r="P22" s="31" t="n">
         <v>5800000</v>
       </c>
-      <c r="Q22" s="28" t="n">
+      <c r="Q22" s="31" t="n">
         <v>4200000</v>
       </c>
-      <c r="R22" s="28" t="n">
+      <c r="R22" s="31" t="n">
         <v>4200000</v>
       </c>
-      <c r="S22" s="28" t="n">
+      <c r="S22" s="31" t="n">
         <v>2840460</v>
       </c>
-      <c r="T22" s="28" t="n">
+      <c r="T22" s="31" t="n">
         <v>1638000</v>
       </c>
-      <c r="U22" s="28" t="n">
+      <c r="U22" s="31" t="n">
         <v>1359540</v>
       </c>
-      <c r="V22" s="28" t="n">
+      <c r="V22" s="31" t="n">
         <v>105000</v>
       </c>
       <c r="W22" s="5" t="inlineStr"/>
@@ -3483,16 +3591,16 @@
           <t>2025-10-31</t>
         </is>
       </c>
-      <c r="Z22" s="29" t="n">
+      <c r="Z22" s="32" t="n">
         <v>45</v>
       </c>
-      <c r="AA22" s="29" t="n">
+      <c r="AA22" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="AB22" s="29" t="n">
+      <c r="AB22" s="32" t="n">
         <v/>
       </c>
-      <c r="AC22" s="29" t="n">
+      <c r="AC22" s="32" t="n">
         <v>11000</v>
       </c>
     </row>
@@ -3568,25 +3676,25 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="P23" s="30" t="n">
+      <c r="P23" s="33" t="n">
         <v>7800000</v>
       </c>
-      <c r="Q23" s="30" t="n">
+      <c r="Q23" s="33" t="n">
         <v>5800000</v>
       </c>
-      <c r="R23" s="30" t="n">
+      <c r="R23" s="33" t="n">
         <v>5800000</v>
       </c>
-      <c r="S23" s="30" t="n">
+      <c r="S23" s="33" t="n">
         <v>3922540</v>
       </c>
-      <c r="T23" s="30" t="n">
+      <c r="T23" s="33" t="n">
         <v>2262000</v>
       </c>
-      <c r="U23" s="30" t="n">
+      <c r="U23" s="33" t="n">
         <v>1877460</v>
       </c>
-      <c r="V23" s="30" t="n">
+      <c r="V23" s="33" t="n">
         <v>145000</v>
       </c>
       <c r="W23" s="7" t="inlineStr"/>
@@ -3596,77 +3704,77 @@
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="Z23" s="31" t="n">
+      <c r="Z23" s="34" t="n">
         <v>32</v>
       </c>
-      <c r="AA23" s="31" t="n">
+      <c r="AA23" s="34" t="n">
         <v>9</v>
       </c>
-      <c r="AB23" s="31" t="n">
+      <c r="AB23" s="34" t="n">
         <v>18</v>
       </c>
-      <c r="AC23" s="31" t="n">
+      <c r="AC23" s="34" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="A24" s="35" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B24" s="32" t="inlineStr"/>
-      <c r="C24" s="32" t="inlineStr">
+      <c r="B24" s="35" t="inlineStr"/>
+      <c r="C24" s="35" t="inlineStr">
         <is>
           <t>TOTAL (20 projects)</t>
         </is>
       </c>
-      <c r="D24" s="32" t="inlineStr"/>
-      <c r="E24" s="32" t="inlineStr"/>
-      <c r="F24" s="32" t="inlineStr"/>
-      <c r="G24" s="32" t="inlineStr"/>
-      <c r="H24" s="32" t="inlineStr"/>
-      <c r="I24" s="32" t="inlineStr"/>
-      <c r="J24" s="32" t="inlineStr"/>
-      <c r="K24" s="32" t="inlineStr"/>
-      <c r="L24" s="32" t="inlineStr"/>
-      <c r="M24" s="32" t="inlineStr"/>
-      <c r="N24" s="32" t="inlineStr"/>
-      <c r="O24" s="32" t="inlineStr"/>
-      <c r="P24" s="33" t="n">
+      <c r="D24" s="35" t="inlineStr"/>
+      <c r="E24" s="35" t="inlineStr"/>
+      <c r="F24" s="35" t="inlineStr"/>
+      <c r="G24" s="35" t="inlineStr"/>
+      <c r="H24" s="35" t="inlineStr"/>
+      <c r="I24" s="35" t="inlineStr"/>
+      <c r="J24" s="35" t="inlineStr"/>
+      <c r="K24" s="35" t="inlineStr"/>
+      <c r="L24" s="35" t="inlineStr"/>
+      <c r="M24" s="35" t="inlineStr"/>
+      <c r="N24" s="35" t="inlineStr"/>
+      <c r="O24" s="35" t="inlineStr"/>
+      <c r="P24" s="36" t="n">
         <v>170600000</v>
       </c>
-      <c r="Q24" s="33" t="n">
+      <c r="Q24" s="36" t="n">
         <v>122500000</v>
       </c>
-      <c r="R24" s="33" t="n">
+      <c r="R24" s="36" t="n">
         <v>122500000</v>
       </c>
-      <c r="S24" s="33" t="n">
+      <c r="S24" s="36" t="n">
         <v>82846750</v>
       </c>
-      <c r="T24" s="33" t="n">
+      <c r="T24" s="36" t="n">
         <v>47775000</v>
       </c>
-      <c r="U24" s="33" t="n">
+      <c r="U24" s="36" t="n">
         <v>39653250</v>
       </c>
-      <c r="V24" s="33" t="n">
+      <c r="V24" s="36" t="n">
         <v>3062500</v>
       </c>
-      <c r="W24" s="32" t="inlineStr"/>
-      <c r="X24" s="32" t="inlineStr"/>
-      <c r="Y24" s="32" t="inlineStr"/>
-      <c r="Z24" s="34" t="n">
+      <c r="W24" s="35" t="inlineStr"/>
+      <c r="X24" s="35" t="inlineStr"/>
+      <c r="Y24" s="35" t="inlineStr"/>
+      <c r="Z24" s="37" t="n">
         <v>864</v>
       </c>
-      <c r="AA24" s="34" t="n">
+      <c r="AA24" s="37" t="n">
         <v>298</v>
       </c>
-      <c r="AB24" s="34" t="n">
+      <c r="AB24" s="37" t="n">
         <v>234</v>
       </c>
-      <c r="AC24" s="34" t="n">
+      <c r="AC24" s="37" t="n">
         <v>198500</v>
       </c>
     </row>
@@ -3691,7 +3799,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3718,16 +3826,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Appendix B: Distress Documentation</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
         </is>
       </c>
     </row>
@@ -5349,41 +5457,41 @@
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="A24" s="35" t="inlineStr">
         <is>
           <t>SUMMARY</t>
         </is>
       </c>
-      <c r="B24" s="32" t="inlineStr">
+      <c r="B24" s="35" t="inlineStr">
         <is>
           <t>20 total projects</t>
         </is>
       </c>
-      <c r="C24" s="32" t="inlineStr"/>
-      <c r="D24" s="32" t="inlineStr"/>
-      <c r="E24" s="32" t="inlineStr">
+      <c r="C24" s="35" t="inlineStr"/>
+      <c r="D24" s="35" t="inlineStr"/>
+      <c r="E24" s="35" t="inlineStr">
         <is>
           <t>20/20</t>
         </is>
       </c>
-      <c r="F24" s="32" t="inlineStr"/>
-      <c r="G24" s="32" t="inlineStr">
+      <c r="F24" s="35" t="inlineStr"/>
+      <c r="G24" s="35" t="inlineStr">
         <is>
           <t>17/20 (85%)</t>
         </is>
       </c>
-      <c r="H24" s="32" t="inlineStr">
+      <c r="H24" s="35" t="inlineStr">
         <is>
           <t>2/20</t>
         </is>
       </c>
-      <c r="I24" s="32" t="inlineStr"/>
-      <c r="J24" s="32" t="inlineStr"/>
-      <c r="K24" s="32" t="inlineStr"/>
-      <c r="L24" s="32" t="inlineStr"/>
-      <c r="M24" s="32" t="inlineStr"/>
-      <c r="N24" s="32" t="inlineStr"/>
-      <c r="O24" s="32" t="inlineStr"/>
+      <c r="I24" s="35" t="inlineStr"/>
+      <c r="J24" s="35" t="inlineStr"/>
+      <c r="K24" s="35" t="inlineStr"/>
+      <c r="L24" s="35" t="inlineStr"/>
+      <c r="M24" s="35" t="inlineStr"/>
+      <c r="N24" s="35" t="inlineStr"/>
+      <c r="O24" s="35" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:O24"/>
@@ -5395,7 +5503,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5415,16 +5523,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Appendix C: Geographic Targeting</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
         </is>
       </c>
     </row>
@@ -5476,25 +5584,25 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="B4" s="29" t="n">
+      <c r="B4" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="28" t="n">
+      <c r="C4" s="31" t="n">
         <v>6500000</v>
       </c>
       <c r="D4" s="17" t="n">
         <v>0.05306122448979592</v>
       </c>
-      <c r="E4" s="29" t="n">
+      <c r="E4" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="29" t="n">
+      <c r="F4" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="29" t="n">
+      <c r="G4" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="29" t="n">
+      <c r="H4" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5504,25 +5612,25 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="B5" s="31" t="n">
+      <c r="B5" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="30" t="n">
+      <c r="C5" s="33" t="n">
         <v>4500000</v>
       </c>
       <c r="D5" s="19" t="n">
         <v>0.03673469387755102</v>
       </c>
-      <c r="E5" s="31" t="n">
+      <c r="E5" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="31" t="n">
+      <c r="F5" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="31" t="n">
+      <c r="G5" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="31" t="n">
+      <c r="H5" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5532,25 +5640,25 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="B6" s="29" t="n">
+      <c r="B6" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="31" t="n">
         <v>4000000</v>
       </c>
       <c r="D6" s="17" t="n">
         <v>0.0326530612244898</v>
       </c>
-      <c r="E6" s="29" t="n">
+      <c r="E6" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="29" t="n">
+      <c r="F6" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="29" t="n">
+      <c r="G6" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="29" t="n">
+      <c r="H6" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5560,25 +5668,25 @@
           <t>GA</t>
         </is>
       </c>
-      <c r="B7" s="31" t="n">
+      <c r="B7" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="30" t="n">
+      <c r="C7" s="33" t="n">
         <v>9000000</v>
       </c>
       <c r="D7" s="19" t="n">
         <v>0.07346938775510205</v>
       </c>
-      <c r="E7" s="31" t="n">
+      <c r="E7" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="31" t="n">
+      <c r="F7" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="31" t="n">
+      <c r="G7" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="31" t="n">
+      <c r="H7" s="34" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5588,25 +5696,25 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="B8" s="29" t="n">
+      <c r="B8" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="31" t="n">
         <v>8500000</v>
       </c>
       <c r="D8" s="17" t="n">
         <v>0.06938775510204082</v>
       </c>
-      <c r="E8" s="29" t="n">
+      <c r="E8" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="29" t="n">
+      <c r="F8" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="29" t="n">
+      <c r="G8" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="29" t="n">
+      <c r="H8" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5616,25 +5724,25 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="B9" s="31" t="n">
+      <c r="B9" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="30" t="n">
+      <c r="C9" s="33" t="n">
         <v>7500000</v>
       </c>
       <c r="D9" s="19" t="n">
         <v>0.06122448979591837</v>
       </c>
-      <c r="E9" s="31" t="n">
+      <c r="E9" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="31" t="n">
+      <c r="F9" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="31" t="n">
+      <c r="G9" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="31" t="n">
+      <c r="H9" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5644,25 +5752,25 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="B10" s="29" t="n">
+      <c r="B10" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="31" t="n">
         <v>6000000</v>
       </c>
       <c r="D10" s="17" t="n">
         <v>0.04897959183673469</v>
       </c>
-      <c r="E10" s="29" t="n">
+      <c r="E10" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="29" t="n">
+      <c r="F10" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="29" t="n">
+      <c r="G10" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="29" t="n">
+      <c r="H10" s="32" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5672,25 +5780,25 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="B11" s="31" t="n">
+      <c r="B11" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="30" t="n">
+      <c r="C11" s="33" t="n">
         <v>4200000</v>
       </c>
       <c r="D11" s="19" t="n">
         <v>0.03428571428571429</v>
       </c>
-      <c r="E11" s="31" t="n">
+      <c r="E11" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="31" t="n">
+      <c r="F11" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="31" t="n">
+      <c r="G11" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="31" t="n">
+      <c r="H11" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5700,25 +5808,25 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="B12" s="29" t="n">
+      <c r="B12" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="31" t="n">
         <v>5000000</v>
       </c>
       <c r="D12" s="17" t="n">
         <v>0.04081632653061224</v>
       </c>
-      <c r="E12" s="29" t="n">
+      <c r="E12" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="29" t="n">
+      <c r="F12" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="29" t="n">
+      <c r="G12" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="29" t="n">
+      <c r="H12" s="32" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5728,25 +5836,25 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="B13" s="31" t="n">
+      <c r="B13" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="30" t="n">
+      <c r="C13" s="33" t="n">
         <v>12300000</v>
       </c>
       <c r="D13" s="19" t="n">
         <v>0.1004081632653061</v>
       </c>
-      <c r="E13" s="31" t="n">
+      <c r="E13" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="31" t="n">
+      <c r="F13" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="31" t="n">
+      <c r="G13" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="31" t="n">
+      <c r="H13" s="34" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5756,25 +5864,25 @@
           <t>MS</t>
         </is>
       </c>
-      <c r="B14" s="29" t="n">
+      <c r="B14" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="31" t="n">
         <v>3200000</v>
       </c>
       <c r="D14" s="17" t="n">
         <v>0.02612244897959184</v>
       </c>
-      <c r="E14" s="29" t="n">
+      <c r="E14" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="29" t="n">
+      <c r="F14" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="29" t="n">
+      <c r="G14" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="29" t="n">
+      <c r="H14" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5784,25 +5892,25 @@
           <t>NC</t>
         </is>
       </c>
-      <c r="B15" s="31" t="n">
+      <c r="B15" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="C15" s="30" t="n">
+      <c r="C15" s="33" t="n">
         <v>5500000</v>
       </c>
       <c r="D15" s="19" t="n">
         <v>0.04489795918367347</v>
       </c>
-      <c r="E15" s="31" t="n">
+      <c r="E15" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="31" t="n">
+      <c r="F15" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="31" t="n">
+      <c r="G15" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="31" t="n">
+      <c r="H15" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5812,25 +5920,25 @@
           <t>NM</t>
         </is>
       </c>
-      <c r="B16" s="29" t="n">
+      <c r="B16" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C16" s="31" t="n">
         <v>5800000</v>
       </c>
       <c r="D16" s="17" t="n">
         <v>0.0473469387755102</v>
       </c>
-      <c r="E16" s="29" t="n">
+      <c r="E16" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="29" t="n">
+      <c r="F16" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="29" t="n">
+      <c r="G16" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="29" t="n">
+      <c r="H16" s="32" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5840,25 +5948,25 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="B17" s="31" t="n">
+      <c r="B17" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="C17" s="30" t="n">
+      <c r="C17" s="33" t="n">
         <v>5000000</v>
       </c>
       <c r="D17" s="19" t="n">
         <v>0.04081632653061224</v>
       </c>
-      <c r="E17" s="31" t="n">
+      <c r="E17" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="31" t="n">
+      <c r="F17" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="31" t="n">
+      <c r="G17" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="31" t="n">
+      <c r="H17" s="34" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5868,25 +5976,25 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="B18" s="29" t="n">
+      <c r="B18" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="28" t="n">
+      <c r="C18" s="31" t="n">
         <v>7500000</v>
       </c>
       <c r="D18" s="17" t="n">
         <v>0.06122448979591837</v>
       </c>
-      <c r="E18" s="29" t="n">
+      <c r="E18" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="29" t="n">
+      <c r="F18" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="29" t="n">
+      <c r="G18" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="29" t="n">
+      <c r="H18" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5896,25 +6004,25 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="B19" s="31" t="n">
+      <c r="B19" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="C19" s="30" t="n">
+      <c r="C19" s="33" t="n">
         <v>8000000</v>
       </c>
       <c r="D19" s="19" t="n">
         <v>0.0653061224489796</v>
       </c>
-      <c r="E19" s="31" t="n">
+      <c r="E19" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="31" t="n">
+      <c r="F19" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="31" t="n">
+      <c r="G19" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="31" t="n">
+      <c r="H19" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5924,25 +6032,25 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="B20" s="29" t="n">
+      <c r="B20" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="C20" s="28" t="n">
+      <c r="C20" s="31" t="n">
         <v>3500000</v>
       </c>
       <c r="D20" s="17" t="n">
         <v>0.02857142857142857</v>
       </c>
-      <c r="E20" s="29" t="n">
+      <c r="E20" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="29" t="n">
+      <c r="F20" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="29" t="n">
+      <c r="G20" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="29" t="n">
+      <c r="H20" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5952,25 +6060,25 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="B21" s="31" t="n">
+      <c r="B21" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="C21" s="30" t="n">
+      <c r="C21" s="33" t="n">
         <v>7000000</v>
       </c>
       <c r="D21" s="19" t="n">
         <v>0.05714285714285714</v>
       </c>
-      <c r="E21" s="31" t="n">
+      <c r="E21" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="31" t="n">
+      <c r="F21" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="31" t="n">
+      <c r="G21" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="31" t="n">
+      <c r="H21" s="34" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5980,53 +6088,53 @@
           <t>WI</t>
         </is>
       </c>
-      <c r="B22" s="29" t="n">
+      <c r="B22" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="C22" s="28" t="n">
+      <c r="C22" s="31" t="n">
         <v>9500000</v>
       </c>
       <c r="D22" s="17" t="n">
         <v>0.07755102040816327</v>
       </c>
-      <c r="E22" s="29" t="n">
+      <c r="E22" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="29" t="n">
+      <c r="F22" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="29" t="n">
+      <c r="G22" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="29" t="n">
+      <c r="H22" s="32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="32" t="inlineStr">
+      <c r="A23" s="35" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B23" s="34" t="n">
+      <c r="B23" s="37" t="n">
         <v>20</v>
       </c>
-      <c r="C23" s="33" t="n">
+      <c r="C23" s="36" t="n">
         <v>122500000</v>
       </c>
-      <c r="D23" s="35" t="n">
+      <c r="D23" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="34" t="n">
+      <c r="E23" s="37" t="n">
         <v>17</v>
       </c>
-      <c r="F23" s="34" t="n">
+      <c r="F23" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="34" t="n">
+      <c r="G23" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="34" t="n">
+      <c r="H23" s="37" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6052,7 +6160,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6082,16 +6190,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Appendix D: Impact Projections</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
         </is>
       </c>
     </row>
@@ -6213,31 +6321,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F4" s="28" t="n">
+      <c r="F4" s="31" t="n">
         <v>8500000</v>
       </c>
-      <c r="G4" s="28" t="n">
+      <c r="G4" s="31" t="n">
         <v>12500000</v>
       </c>
-      <c r="H4" s="29" t="n">
+      <c r="H4" s="32" t="n">
         <v>52</v>
       </c>
-      <c r="I4" s="29" t="n">
+      <c r="I4" s="32" t="n">
         <v>18</v>
       </c>
-      <c r="J4" s="29" t="n">
+      <c r="J4" s="32" t="n">
         <v>70</v>
       </c>
-      <c r="K4" s="28" t="n">
+      <c r="K4" s="31" t="n">
         <v>240385</v>
       </c>
-      <c r="L4" s="28" t="n">
+      <c r="L4" s="31" t="n">
         <v>163462</v>
       </c>
-      <c r="M4" s="29" t="n">
+      <c r="M4" s="32" t="n">
         <v/>
       </c>
-      <c r="N4" s="29" t="n">
+      <c r="N4" s="32" t="n">
         <v>24000</v>
       </c>
       <c r="O4" s="5" t="inlineStr">
@@ -6287,31 +6395,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F5" s="30" t="n">
+      <c r="F5" s="33" t="n">
         <v>7000000</v>
       </c>
-      <c r="G5" s="30" t="n">
+      <c r="G5" s="33" t="n">
         <v>9800000</v>
       </c>
-      <c r="H5" s="31" t="n">
+      <c r="H5" s="34" t="n">
         <v>38</v>
       </c>
-      <c r="I5" s="31" t="n">
+      <c r="I5" s="34" t="n">
         <v>22</v>
       </c>
-      <c r="J5" s="31" t="n">
+      <c r="J5" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="K5" s="30" t="n">
+      <c r="K5" s="33" t="n">
         <v>257895</v>
       </c>
-      <c r="L5" s="30" t="n">
+      <c r="L5" s="33" t="n">
         <v>184211</v>
       </c>
-      <c r="M5" s="31" t="n">
+      <c r="M5" s="34" t="n">
         <v/>
       </c>
-      <c r="N5" s="31" t="n">
+      <c r="N5" s="34" t="n">
         <v>0</v>
       </c>
       <c r="O5" s="7" t="inlineStr">
@@ -6361,31 +6469,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="31" t="n">
         <v>5000000</v>
       </c>
-      <c r="G6" s="28" t="n">
+      <c r="G6" s="31" t="n">
         <v>7200000</v>
       </c>
-      <c r="H6" s="29" t="n">
+      <c r="H6" s="32" t="n">
         <v>65</v>
       </c>
-      <c r="I6" s="29" t="n">
+      <c r="I6" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="J6" s="29" t="n">
+      <c r="J6" s="32" t="n">
         <v>73</v>
       </c>
-      <c r="K6" s="28" t="n">
+      <c r="K6" s="31" t="n">
         <v>110769</v>
       </c>
-      <c r="L6" s="28" t="n">
+      <c r="L6" s="31" t="n">
         <v>76923</v>
       </c>
-      <c r="M6" s="29" t="n">
+      <c r="M6" s="32" t="n">
         <v/>
       </c>
-      <c r="N6" s="29" t="n">
+      <c r="N6" s="32" t="n">
         <v>18000</v>
       </c>
       <c r="O6" s="5" t="inlineStr">
@@ -6435,31 +6543,31 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F7" s="33" t="n">
         <v>4500000</v>
       </c>
-      <c r="G7" s="30" t="n">
+      <c r="G7" s="33" t="n">
         <v>6000000</v>
       </c>
-      <c r="H7" s="31" t="n">
+      <c r="H7" s="34" t="n">
         <v>80</v>
       </c>
-      <c r="I7" s="31" t="n">
+      <c r="I7" s="34" t="n">
         <v>25</v>
       </c>
-      <c r="J7" s="31" t="n">
+      <c r="J7" s="34" t="n">
         <v>105</v>
       </c>
-      <c r="K7" s="30" t="n">
+      <c r="K7" s="33" t="n">
         <v>75000</v>
       </c>
-      <c r="L7" s="30" t="n">
+      <c r="L7" s="33" t="n">
         <v>56250</v>
       </c>
-      <c r="M7" s="31" t="n">
+      <c r="M7" s="34" t="n">
         <v/>
       </c>
-      <c r="N7" s="31" t="n">
+      <c r="N7" s="34" t="n">
         <v>0</v>
       </c>
       <c r="O7" s="7" t="inlineStr">
@@ -6509,31 +6617,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="31" t="n">
         <v>7500000</v>
       </c>
-      <c r="G8" s="28" t="n">
+      <c r="G8" s="31" t="n">
         <v>10000000</v>
       </c>
-      <c r="H8" s="29" t="n">
+      <c r="H8" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="I8" s="29" t="n">
+      <c r="I8" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="J8" s="29" t="n">
+      <c r="J8" s="32" t="n">
         <v>72</v>
       </c>
-      <c r="K8" s="28" t="n">
+      <c r="K8" s="31" t="n">
         <v>238095</v>
       </c>
-      <c r="L8" s="28" t="n">
+      <c r="L8" s="31" t="n">
         <v>178571</v>
       </c>
-      <c r="M8" s="29" t="n">
+      <c r="M8" s="32" t="n">
         <v/>
       </c>
-      <c r="N8" s="29" t="n">
+      <c r="N8" s="32" t="n">
         <v>20000</v>
       </c>
       <c r="O8" s="5" t="inlineStr">
@@ -6583,31 +6691,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F9" s="30" t="n">
+      <c r="F9" s="33" t="n">
         <v>9000000</v>
       </c>
-      <c r="G9" s="30" t="n">
+      <c r="G9" s="33" t="n">
         <v>14000000</v>
       </c>
-      <c r="H9" s="31" t="n">
+      <c r="H9" s="34" t="n">
         <v>15</v>
       </c>
-      <c r="I9" s="31" t="n">
+      <c r="I9" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="J9" s="31" t="n">
+      <c r="J9" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="K9" s="30" t="n">
+      <c r="K9" s="33" t="n">
         <v>933333</v>
       </c>
-      <c r="L9" s="30" t="n">
+      <c r="L9" s="33" t="n">
         <v>600000</v>
       </c>
-      <c r="M9" s="31" t="n">
+      <c r="M9" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="N9" s="31" t="n">
+      <c r="N9" s="34" t="n">
         <v>0</v>
       </c>
       <c r="O9" s="7" t="inlineStr">
@@ -6657,31 +6765,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="31" t="n">
         <v>4000000</v>
       </c>
-      <c r="G10" s="28" t="n">
+      <c r="G10" s="31" t="n">
         <v>5500000</v>
       </c>
-      <c r="H10" s="29" t="n">
+      <c r="H10" s="32" t="n">
         <v>28</v>
       </c>
-      <c r="I10" s="29" t="n">
+      <c r="I10" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="J10" s="29" t="n">
+      <c r="J10" s="32" t="n">
         <v>38</v>
       </c>
-      <c r="K10" s="28" t="n">
+      <c r="K10" s="31" t="n">
         <v>196429</v>
       </c>
-      <c r="L10" s="28" t="n">
+      <c r="L10" s="31" t="n">
         <v>142857</v>
       </c>
-      <c r="M10" s="29" t="n">
+      <c r="M10" s="32" t="n">
         <v/>
       </c>
-      <c r="N10" s="29" t="n">
+      <c r="N10" s="32" t="n">
         <v>12000</v>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -6731,31 +6839,31 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="F11" s="30" t="n">
+      <c r="F11" s="33" t="n">
         <v>8000000</v>
       </c>
-      <c r="G11" s="30" t="n">
+      <c r="G11" s="33" t="n">
         <v>11000000</v>
       </c>
-      <c r="H11" s="31" t="n">
+      <c r="H11" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="I11" s="31" t="n">
+      <c r="I11" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="J11" s="31" t="n">
+      <c r="J11" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="K11" s="30" t="n">
+      <c r="K11" s="33" t="n">
         <v>200000</v>
       </c>
-      <c r="L11" s="30" t="n">
+      <c r="L11" s="33" t="n">
         <v>145455</v>
       </c>
-      <c r="M11" s="31" t="n">
+      <c r="M11" s="34" t="n">
         <v/>
       </c>
-      <c r="N11" s="31" t="n">
+      <c r="N11" s="34" t="n">
         <v>22000</v>
       </c>
       <c r="O11" s="7" t="inlineStr">
@@ -6805,31 +6913,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F12" s="28" t="n">
+      <c r="F12" s="31" t="n">
         <v>6000000</v>
       </c>
-      <c r="G12" s="28" t="n">
+      <c r="G12" s="31" t="n">
         <v>8200000</v>
       </c>
-      <c r="H12" s="29" t="n">
+      <c r="H12" s="32" t="n">
         <v>35</v>
       </c>
-      <c r="I12" s="29" t="n">
+      <c r="I12" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="J12" s="29" t="n">
+      <c r="J12" s="32" t="n">
         <v>43</v>
       </c>
-      <c r="K12" s="28" t="n">
+      <c r="K12" s="31" t="n">
         <v>234286</v>
       </c>
-      <c r="L12" s="28" t="n">
+      <c r="L12" s="31" t="n">
         <v>171429</v>
       </c>
-      <c r="M12" s="29" t="n">
+      <c r="M12" s="32" t="n">
         <v/>
       </c>
-      <c r="N12" s="29" t="n">
+      <c r="N12" s="32" t="n">
         <v>16000</v>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -6879,31 +6987,31 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="F13" s="30" t="n">
+      <c r="F13" s="33" t="n">
         <v>3500000</v>
       </c>
-      <c r="G13" s="30" t="n">
+      <c r="G13" s="33" t="n">
         <v>4800000</v>
       </c>
-      <c r="H13" s="31" t="n">
+      <c r="H13" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="I13" s="31" t="n">
+      <c r="I13" s="34" t="n">
         <v>15</v>
       </c>
-      <c r="J13" s="31" t="n">
+      <c r="J13" s="34" t="n">
         <v>105</v>
       </c>
-      <c r="K13" s="30" t="n">
+      <c r="K13" s="33" t="n">
         <v>53333</v>
       </c>
-      <c r="L13" s="30" t="n">
+      <c r="L13" s="33" t="n">
         <v>38889</v>
       </c>
-      <c r="M13" s="31" t="n">
+      <c r="M13" s="34" t="n">
         <v/>
       </c>
-      <c r="N13" s="31" t="n">
+      <c r="N13" s="34" t="n">
         <v>0</v>
       </c>
       <c r="O13" s="7" t="inlineStr">
@@ -6953,31 +7061,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F14" s="28" t="n">
+      <c r="F14" s="31" t="n">
         <v>9500000</v>
       </c>
-      <c r="G14" s="28" t="n">
+      <c r="G14" s="31" t="n">
         <v>13500000</v>
       </c>
-      <c r="H14" s="29" t="n">
+      <c r="H14" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="I14" s="29" t="n">
+      <c r="I14" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="J14" s="29" t="n">
+      <c r="J14" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="K14" s="28" t="n">
+      <c r="K14" s="31" t="n">
         <v>1125000</v>
       </c>
-      <c r="L14" s="28" t="n">
+      <c r="L14" s="31" t="n">
         <v>791667</v>
       </c>
-      <c r="M14" s="29" t="n">
+      <c r="M14" s="32" t="n">
         <v>64</v>
       </c>
-      <c r="N14" s="29" t="n">
+      <c r="N14" s="32" t="n">
         <v>0</v>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -7027,31 +7135,31 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="F15" s="30" t="n">
+      <c r="F15" s="33" t="n">
         <v>3800000</v>
       </c>
-      <c r="G15" s="30" t="n">
+      <c r="G15" s="33" t="n">
         <v>5000000</v>
       </c>
-      <c r="H15" s="31" t="n">
+      <c r="H15" s="34" t="n">
         <v>22</v>
       </c>
-      <c r="I15" s="31" t="n">
+      <c r="I15" s="34" t="n">
         <v>6</v>
       </c>
-      <c r="J15" s="31" t="n">
+      <c r="J15" s="34" t="n">
         <v>28</v>
       </c>
-      <c r="K15" s="30" t="n">
+      <c r="K15" s="33" t="n">
         <v>227273</v>
       </c>
-      <c r="L15" s="30" t="n">
+      <c r="L15" s="33" t="n">
         <v>172727</v>
       </c>
-      <c r="M15" s="31" t="n">
+      <c r="M15" s="34" t="n">
         <v/>
       </c>
-      <c r="N15" s="31" t="n">
+      <c r="N15" s="34" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="7" t="inlineStr">
@@ -7101,31 +7209,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F16" s="28" t="n">
+      <c r="F16" s="31" t="n">
         <v>5500000</v>
       </c>
-      <c r="G16" s="28" t="n">
+      <c r="G16" s="31" t="n">
         <v>7500000</v>
       </c>
-      <c r="H16" s="29" t="n">
+      <c r="H16" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="I16" s="29" t="n">
+      <c r="I16" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="J16" s="29" t="n">
+      <c r="J16" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="K16" s="28" t="n">
+      <c r="K16" s="31" t="n">
         <v>250000</v>
       </c>
-      <c r="L16" s="28" t="n">
+      <c r="L16" s="31" t="n">
         <v>183333</v>
       </c>
-      <c r="M16" s="29" t="n">
+      <c r="M16" s="32" t="n">
         <v/>
       </c>
-      <c r="N16" s="29" t="n">
+      <c r="N16" s="32" t="n">
         <v>14000</v>
       </c>
       <c r="O16" s="5" t="inlineStr">
@@ -7175,31 +7283,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F17" s="30" t="n">
+      <c r="F17" s="33" t="n">
         <v>6500000</v>
       </c>
-      <c r="G17" s="30" t="n">
+      <c r="G17" s="33" t="n">
         <v>9000000</v>
       </c>
-      <c r="H17" s="31" t="n">
+      <c r="H17" s="34" t="n">
         <v>48</v>
       </c>
-      <c r="I17" s="31" t="n">
+      <c r="I17" s="34" t="n">
         <v>25</v>
       </c>
-      <c r="J17" s="31" t="n">
+      <c r="J17" s="34" t="n">
         <v>73</v>
       </c>
-      <c r="K17" s="30" t="n">
+      <c r="K17" s="33" t="n">
         <v>187500</v>
       </c>
-      <c r="L17" s="30" t="n">
+      <c r="L17" s="33" t="n">
         <v>135417</v>
       </c>
-      <c r="M17" s="31" t="n">
+      <c r="M17" s="34" t="n">
         <v/>
       </c>
-      <c r="N17" s="31" t="n">
+      <c r="N17" s="34" t="n">
         <v>18500</v>
       </c>
       <c r="O17" s="7" t="inlineStr">
@@ -7249,31 +7357,31 @@
           <t>Operating Business</t>
         </is>
       </c>
-      <c r="F18" s="28" t="n">
+      <c r="F18" s="31" t="n">
         <v>5000000</v>
       </c>
-      <c r="G18" s="28" t="n">
+      <c r="G18" s="31" t="n">
         <v>6500000</v>
       </c>
-      <c r="H18" s="29" t="n">
+      <c r="H18" s="32" t="n">
         <v>110</v>
       </c>
-      <c r="I18" s="29" t="n">
+      <c r="I18" s="32" t="n">
         <v>45</v>
       </c>
-      <c r="J18" s="29" t="n">
+      <c r="J18" s="32" t="n">
         <v>155</v>
       </c>
-      <c r="K18" s="28" t="n">
+      <c r="K18" s="31" t="n">
         <v>59091</v>
       </c>
-      <c r="L18" s="28" t="n">
+      <c r="L18" s="31" t="n">
         <v>45455</v>
       </c>
-      <c r="M18" s="29" t="n">
+      <c r="M18" s="32" t="n">
         <v/>
       </c>
-      <c r="N18" s="29" t="n">
+      <c r="N18" s="32" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="5" t="inlineStr">
@@ -7323,31 +7431,31 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="F19" s="30" t="n">
+      <c r="F19" s="33" t="n">
         <v>7500000</v>
       </c>
-      <c r="G19" s="30" t="n">
+      <c r="G19" s="33" t="n">
         <v>10500000</v>
       </c>
-      <c r="H19" s="31" t="n">
+      <c r="H19" s="34" t="n">
         <v>35</v>
       </c>
-      <c r="I19" s="31" t="n">
+      <c r="I19" s="34" t="n">
         <v>10</v>
       </c>
-      <c r="J19" s="31" t="n">
+      <c r="J19" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="K19" s="30" t="n">
+      <c r="K19" s="33" t="n">
         <v>300000</v>
       </c>
-      <c r="L19" s="30" t="n">
+      <c r="L19" s="33" t="n">
         <v>214286</v>
       </c>
-      <c r="M19" s="31" t="n">
+      <c r="M19" s="34" t="n">
         <v>24</v>
       </c>
-      <c r="N19" s="31" t="n">
+      <c r="N19" s="34" t="n">
         <v>20000</v>
       </c>
       <c r="O19" s="7" t="inlineStr">
@@ -7397,31 +7505,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F20" s="28" t="n">
+      <c r="F20" s="31" t="n">
         <v>3200000</v>
       </c>
-      <c r="G20" s="28" t="n">
+      <c r="G20" s="31" t="n">
         <v>4200000</v>
       </c>
-      <c r="H20" s="29" t="n">
+      <c r="H20" s="32" t="n">
         <v>20</v>
       </c>
-      <c r="I20" s="29" t="n">
+      <c r="I20" s="32" t="n">
         <v>15</v>
       </c>
-      <c r="J20" s="29" t="n">
+      <c r="J20" s="32" t="n">
         <v>35</v>
       </c>
-      <c r="K20" s="28" t="n">
+      <c r="K20" s="31" t="n">
         <v>210000</v>
       </c>
-      <c r="L20" s="28" t="n">
+      <c r="L20" s="31" t="n">
         <v>160000</v>
       </c>
-      <c r="M20" s="29" t="n">
+      <c r="M20" s="32" t="n">
         <v/>
       </c>
-      <c r="N20" s="29" t="n">
+      <c r="N20" s="32" t="n">
         <v>8000</v>
       </c>
       <c r="O20" s="5" t="inlineStr">
@@ -7471,31 +7579,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F21" s="30" t="n">
+      <c r="F21" s="33" t="n">
         <v>8500000</v>
       </c>
-      <c r="G21" s="30" t="n">
+      <c r="G21" s="33" t="n">
         <v>11800000</v>
       </c>
-      <c r="H21" s="31" t="n">
+      <c r="H21" s="34" t="n">
         <v>10</v>
       </c>
-      <c r="I21" s="31" t="n">
+      <c r="I21" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="J21" s="31" t="n">
+      <c r="J21" s="34" t="n">
         <v>13</v>
       </c>
-      <c r="K21" s="30" t="n">
+      <c r="K21" s="33" t="n">
         <v>1180000</v>
       </c>
-      <c r="L21" s="30" t="n">
+      <c r="L21" s="33" t="n">
         <v>850000</v>
       </c>
-      <c r="M21" s="31" t="n">
+      <c r="M21" s="34" t="n">
         <v>56</v>
       </c>
-      <c r="N21" s="31" t="n">
+      <c r="N21" s="34" t="n">
         <v>0</v>
       </c>
       <c r="O21" s="7" t="inlineStr">
@@ -7545,31 +7653,31 @@
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="F22" s="28" t="n">
+      <c r="F22" s="31" t="n">
         <v>4200000</v>
       </c>
-      <c r="G22" s="28" t="n">
+      <c r="G22" s="31" t="n">
         <v>5800000</v>
       </c>
-      <c r="H22" s="29" t="n">
+      <c r="H22" s="32" t="n">
         <v>45</v>
       </c>
-      <c r="I22" s="29" t="n">
+      <c r="I22" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="J22" s="29" t="n">
+      <c r="J22" s="32" t="n">
         <v>53</v>
       </c>
-      <c r="K22" s="28" t="n">
+      <c r="K22" s="31" t="n">
         <v>128889</v>
       </c>
-      <c r="L22" s="28" t="n">
+      <c r="L22" s="31" t="n">
         <v>93333</v>
       </c>
-      <c r="M22" s="29" t="n">
+      <c r="M22" s="32" t="n">
         <v/>
       </c>
-      <c r="N22" s="29" t="n">
+      <c r="N22" s="32" t="n">
         <v>11000</v>
       </c>
       <c r="O22" s="5" t="inlineStr">
@@ -7619,31 +7727,31 @@
           <t>Mixed Use</t>
         </is>
       </c>
-      <c r="F23" s="30" t="n">
+      <c r="F23" s="33" t="n">
         <v>5800000</v>
       </c>
-      <c r="G23" s="30" t="n">
+      <c r="G23" s="33" t="n">
         <v>7800000</v>
       </c>
-      <c r="H23" s="31" t="n">
+      <c r="H23" s="34" t="n">
         <v>32</v>
       </c>
-      <c r="I23" s="31" t="n">
+      <c r="I23" s="34" t="n">
         <v>9</v>
       </c>
-      <c r="J23" s="31" t="n">
+      <c r="J23" s="34" t="n">
         <v>41</v>
       </c>
-      <c r="K23" s="30" t="n">
+      <c r="K23" s="33" t="n">
         <v>243750</v>
       </c>
-      <c r="L23" s="30" t="n">
+      <c r="L23" s="33" t="n">
         <v>181250</v>
       </c>
-      <c r="M23" s="31" t="n">
+      <c r="M23" s="34" t="n">
         <v>18</v>
       </c>
-      <c r="N23" s="31" t="n">
+      <c r="N23" s="34" t="n">
         <v>15000</v>
       </c>
       <c r="O23" s="7" t="inlineStr">
@@ -7668,50 +7776,50 @@
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="A24" s="35" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B24" s="32" t="inlineStr">
+      <c r="B24" s="35" t="inlineStr">
         <is>
           <t>20 Projects</t>
         </is>
       </c>
-      <c r="C24" s="32" t="inlineStr"/>
-      <c r="D24" s="32" t="inlineStr"/>
-      <c r="E24" s="32" t="inlineStr"/>
-      <c r="F24" s="33" t="n">
+      <c r="C24" s="35" t="inlineStr"/>
+      <c r="D24" s="35" t="inlineStr"/>
+      <c r="E24" s="35" t="inlineStr"/>
+      <c r="F24" s="36" t="n">
         <v>122500000</v>
       </c>
-      <c r="G24" s="33" t="n">
+      <c r="G24" s="36" t="n">
         <v>170600000</v>
       </c>
-      <c r="H24" s="34" t="n">
+      <c r="H24" s="37" t="n">
         <v>864</v>
       </c>
-      <c r="I24" s="34" t="n">
+      <c r="I24" s="37" t="n">
         <v>298</v>
       </c>
-      <c r="J24" s="34" t="n">
+      <c r="J24" s="37" t="n">
         <v>1162</v>
       </c>
-      <c r="K24" s="33" t="n">
+      <c r="K24" s="36" t="n">
         <v>197454</v>
       </c>
-      <c r="L24" s="33" t="n">
+      <c r="L24" s="36" t="n">
         <v>141782</v>
       </c>
-      <c r="M24" s="34" t="n">
+      <c r="M24" s="37" t="n">
         <v>234</v>
       </c>
-      <c r="N24" s="34" t="n">
+      <c r="N24" s="37" t="n">
         <v>198500</v>
       </c>
-      <c r="O24" s="32" t="inlineStr"/>
-      <c r="P24" s="32" t="inlineStr"/>
-      <c r="Q24" s="32" t="inlineStr"/>
-      <c r="R24" s="32" t="inlineStr"/>
+      <c r="O24" s="35" t="inlineStr"/>
+      <c r="P24" s="35" t="inlineStr"/>
+      <c r="Q24" s="35" t="inlineStr"/>
+      <c r="R24" s="35" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:R24"/>
@@ -7723,7 +7831,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7743,16 +7851,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Section D: Investor Commitments</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
         </is>
       </c>
     </row>
@@ -7882,27 +7990,27 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="32" t="inlineStr">
+    <row r="6" ht="120" customHeight="1">
+      <c r="A6" s="35" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B6" s="32" t="inlineStr"/>
-      <c r="C6" s="32" t="inlineStr"/>
-      <c r="D6" s="32" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr"/>
+      <c r="C6" s="35" t="inlineStr"/>
+      <c r="D6" s="35" t="inlineStr">
         <is>
           <t>[CDE TO COMPLETE]</t>
         </is>
       </c>
-      <c r="E6" s="32" t="inlineStr"/>
-      <c r="F6" s="32" t="inlineStr"/>
-      <c r="G6" s="32" t="inlineStr">
+      <c r="E6" s="35" t="inlineStr"/>
+      <c r="F6" s="35" t="inlineStr"/>
+      <c r="G6" s="35" t="inlineStr">
         <is>
           <t>[CDE TO COMPLETE: This table is a blank form. nmtc-application-builder holds no investor data for your CDE and supplies no figure in it — not a name, a type, a CRA obligation, a commitment amount, a credit price or a status, and not the number of rows. Add one row per investor you can name and defend to the CDFI Fund, and delete any row you cannot.]</t>
         </is>
       </c>
-      <c r="H6" s="32" t="inlineStr">
+      <c r="H6" s="35" t="inlineStr">
         <is>
           <t>[CDE TO COMPLETE]</t>
         </is>
@@ -7918,7 +8026,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7936,16 +8044,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Appendix E: CDE Track Record</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-17</t>
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
         </is>
       </c>
     </row>
@@ -7982,10 +8090,10 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="36" t="n">
+      <c r="A4" s="39" t="n">
         <v>2019</v>
       </c>
-      <c r="B4" s="28" t="n">
+      <c r="B4" s="31" t="n">
         <v>40000000</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -8006,10 +8114,10 @@
       <c r="F4" s="5" t="inlineStr"/>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="37" t="n">
+      <c r="A5" s="40" t="n">
         <v>2021</v>
       </c>
-      <c r="B5" s="30" t="n">
+      <c r="B5" s="33" t="n">
         <v>55000000</v>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -8030,10 +8138,10 @@
       <c r="F5" s="7" t="inlineStr"/>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="36" t="n">
+      <c r="A6" s="39" t="n">
         <v>2023</v>
       </c>
-      <c r="B6" s="28" t="n">
+      <c r="B6" s="31" t="n">
         <v>60000000</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -8054,26 +8162,26 @@
       <c r="F6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="32" t="inlineStr">
+      <c r="A7" s="35" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B7" s="33" t="n">
+      <c r="B7" s="36" t="n">
         <v>155000000</v>
       </c>
-      <c r="C7" s="32" t="inlineStr">
+      <c r="C7" s="35" t="inlineStr">
         <is>
           <t>2 rounds fully deployed</t>
         </is>
       </c>
-      <c r="D7" s="32" t="inlineStr">
+      <c r="D7" s="35" t="inlineStr">
         <is>
           <t>7 states</t>
         </is>
       </c>
-      <c r="E7" s="32" t="inlineStr"/>
-      <c r="F7" s="32" t="inlineStr">
+      <c r="E7" s="35" t="inlineStr"/>
+      <c r="F7" s="35" t="inlineStr">
         <is>
           <t>$155,000,000 total prior allocation</t>
         </is>

</xml_diff>

<commit_message>
Deployed c709d79 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -894,7 +894,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>CY2025  |  Prepared: August 19, 2026  |  Readiness Grade: A (86.6/100)</t>
+          <t>CY2025  |  Prepared: August 20, 2026  |  Readiness Grade: A (86.6/100)</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-19</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-20</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>Every distress share in this document is a share of QEI. nmtc-application-builder computes neither QLICI-denominated figure — it reads this pipeline's QLICI amounts only to print them in Appendix A and to check that each is no larger than its QEI — so no figure in this document answers either commitment, and none may be presented to the CDFI Fund as doing so. WHICH OF THE CDE'S QUALIFYING ROUTES ARE VISIBLE HERE: this package carries a per-project field for 5 of the 14 distinct area types Question 25 lists, and they do NOT share one provenance, so each is stated with its own.</t>
+          <t>Every distress share in this document is a share of QEI. nmtc-application-builder computes neither QLICI-denominated figure — it reads this pipeline's QLICI amounts only to print them in Appendix A and to check that each is no larger than its QEI — so no figure in this document answers either commitment, and none may be presented to the CDFI Fund as doing so. WHICH OF THE CDE'S QUALIFYING ROUTES ARE VISIBLE HERE: this package carries a per-project field for 6 of the 14 distinct area types Question 25 lists, and they do NOT share one provenance, so each is stated with its own.</t>
         </is>
       </c>
     </row>
@@ -1230,14 +1230,14 @@
     <row r="8" ht="98" customHeight="1">
       <c r="A8" s="28" t="inlineStr">
         <is>
-          <t>NMTC Native Areas and U.S. territory: CDE-DECLARED AND TOOL-UNVERIFIED — nothing in this package checks either one, and a Native Area determination is a spatial intersection against the Fund's CIMS map rather than a tract-keyed lookup this package could perform (U.S. territory is the CDE's own word; the Application's U.S. Island Areas is a specific list of five). It carries NOTHING for Non-Metropolitan Counties, nothing for Targeted Populations, and nothing for any of items 6-12; it computes no multi-indicia measure at all. Holding those fields is not a partial answer to Question 25 and must not be read as one: the commitment is a share of QLICI DOLLARS, this package weights nothing by QLICI dollars, and a flag that enters no denominator contributes nothing to a share.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
+          <t>NMTC Native Areas and U.S. territory: CDE-DECLARED AND TOOL-UNVERIFIED — nothing in this package checks either one, and a Native Area determination is a spatial intersection against the Fund's CIMS map rather than a tract-keyed lookup this package could perform (U.S. territory is the CDE's own word; the Application's U.S. Island Areas is a specific list of five). Non-Metropolitan Counties: TOOL-VERIFIED AND TRI-STATE — the OMB designation is read for the same geocoded tract, and a project the lookup could not resolve is recorded as undetermined rather than as metropolitan, so no project is counted in a county type it was never determined to be in. It carries NOTHING for Targeted Populations and nothing for any of items 6-12; it computes no multi-indicia measure at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1">
       <c r="A9" s="28" t="inlineStr">
         <is>
-          <t>Deep Distress is a strict subset of severe distress, so the severe-distress share already includes the deep-distress share. The CDE must compute both QLICI-denominated shares from its own QLICI amounts, against the Application's own area lists, before stating either commitment. (The CY 2026 NOAA is not yet published.)</t>
+          <t>Holding those fields is not a partial answer to Question 25 and must not be read as one: the commitment is a share of QLICI DOLLARS, this package weights nothing by QLICI dollars, and a flag that enters no denominator contributes nothing to a share. Deep Distress is a strict subset of severe distress, so the severe-distress share already includes the deep-distress share. The CDE must compute both QLICI-denominated shares from its own QLICI amounts, against the Application's own area lists, before stating either commitment. (The CY 2026 NOAA is not yet published.)</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1306,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
         </is>
       </c>
     </row>
@@ -6199,7 +6199,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
         </is>
       </c>
     </row>
@@ -8053,7 +8053,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 0cb79e2 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -9,20 +9,21 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary Dashboard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q25 Basis Note" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Detail" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distress Documentation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geographic Targeting" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Projections" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investor Commitments" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track Record" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round Provenance" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Detail" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distress Documentation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geographic Targeting" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Projections" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investor Commitments" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track Record" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pipeline Detail'!$A$3:$AC$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Distress Documentation'!$A$3:$O$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Geographic Targeting'!$A$3:$H$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Impact Projections'!$A$3:$R$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Investor Commitments'!$A$3:$H$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Track Record'!$A$3:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pipeline Detail'!$A$3:$AC$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Distress Documentation'!$A$3:$O$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Geographic Targeting'!$A$3:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Impact Projections'!$A$3:$R$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Investor Commitments'!$A$3:$H$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Track Record'!$A$3:$F$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -894,7 +895,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>CY2025  |  Prepared: August 20, 2026  |  Readiness Grade: A (86.6/100)</t>
+          <t>CY2025  |  Prepared: August 21, 2026  |  Readiness Grade: A (86.6/100)</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1124,7 @@
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-20</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-21</t>
         </is>
       </c>
     </row>
@@ -1262,6 +1263,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>WHICH ROUND THIS WORKBOOK IS BASED ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>This applies to every round-specific citation in this workbook, including the 'Q25 Basis Note' sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="70" customHeight="1">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>WHICH ROUND THIS IS BASED ON. This tool encodes the CY 2024-2025 NMTC Allocation Application, which is the most recent PUBLISHED Application and is closed and awarded (it opened 19 Nov 2024, closed 29 Jan 2025, and was awarded 23 Dec 2025 with $10 billion in allocation authority). The CY 2026 Allocation Application and NOAA are NOT YET PUBLISHED: the CDFI Fund has announced that CY 2026 will make $5 billion available — half the prior round — and that it will publish the round's Application Materials when the round opens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="84" customHeight="1">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>USE THIS, AND THEN RE-CHECK IT. The CY 2024-2025 Application is a real federal instrument and is the right basis to prepare against today; nothing here is unreliable. But it is a PROXY for the CY 2026 instrument, not that instrument, so every round-specific figure in this document must be re-verified against the CY 2026 materials once the Fund releases them — specifically: the allocation authority and the number of awards available; the CDE certification deadline for eligibility; Question 25's QLICI-denominated commitment levels, its area-type lists and its ladder; Question 22's QLICI-denominated Non-Metropolitan minimum and maximum; Question 15's product-flexibility ladder; the scoring thresholds in the Review Process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>SEPARATELY, AND SOONER: to be eligible to apply in CY 2026, an organization must either already be a certified CDE as of the NOAA's Federal Register publication date, or have submitted its CDE Certification Application through AMIS by 11:59 p.m. ET on August 31, 2026. That deadline is not a figure this tool computes and it does not move with anything in this document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="84" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>AND IF YOU ARE A PRIOR ALLOCATEE, A THIRD OBLIGATION FALLS ON THE SAME DATE: any prior Allocatee that requires action by the CDFI Fund — certifying a Subsidiary entity as a CDE, or adding a Subsidiary CDE to an Allocation Agreement — in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA must submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on August 31, 2026. Full eligibility information, including the QEI issuance thresholds themselves, comes with the NOAA when it publishes. Verified against cdfifund.gov on 2026-08-20.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A7:F7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AW24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1306,7 +1379,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3872,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3835,7 +3908,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
         </is>
       </c>
     </row>
@@ -5503,7 +5576,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5532,7 +5605,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6233,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6199,7 +6272,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
         </is>
       </c>
     </row>
@@ -7831,7 +7904,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7860,7 +7933,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
         </is>
       </c>
     </row>
@@ -8026,7 +8099,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8053,7 +8126,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-20</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed fde3eca with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -892,10 +892,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>CY2025  |  Prepared: August 21, 2026  |  Readiness Grade: A (86.6/100)</t>
+          <t>CY2025  |  Prepared: August 21, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed e483ae1 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>CY2025  |  Prepared: August 21, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
+          <t>CY2025  |  Prepared: August 22, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-21</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-22</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
         </is>
       </c>
     </row>
@@ -3908,7 +3908,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
         </is>
       </c>
     </row>
@@ -5605,7 +5605,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
         </is>
       </c>
     </row>
@@ -6272,7 +6272,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
         </is>
       </c>
     </row>
@@ -7933,7 +7933,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
         </is>
       </c>
     </row>
@@ -8126,7 +8126,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-21</t>
+          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 1313aea with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>CY2025  |  Prepared: August 22, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
+          <t>Application round not specified  |  Prepared: August 23, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC CY2025 — Generated 2026-08-22</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3908,7 +3908,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -5605,7 +5605,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -6272,7 +6272,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -7933,7 +7933,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -8126,7 +8126,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  CY2025  |  Generated 2026-08-22</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
         </is>
       </c>
     </row>

</xml_diff>